<commit_message>
Leave the mortgage and auto loan out of liquid net worth
Liquid net worth subtracted every debt, so a homeowner saw a large
negative figure driven by the mortgage while the home itself was left
out. It now subtracts only student loans, credit cards and other debt;
the mortgage and auto loan are excluded along with the home and car
that secure them. In the sample data this moves liquid net worth from
-$277,000 to +$33,000.

The Liquid column on Accounts and Lists now also marks the debts that
count against liquid assets, and the Dashboard note explains the rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171gMz8tZxkRy1j67VNEeC6
</commit_message>
<xml_diff>
--- a/public/templates/net-worth-dashboard.xlsx
+++ b/public/templates/net-worth-dashboard.xlsx
@@ -117,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +146,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1055,9 +1058,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Liquid net worth counts cash and taxable investing, minus all debts.</t>
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Liquid net worth: cash and taxable investing, minus debts other than the mortgage and auto loan.</t>
         </is>
       </c>
       <c r="E13" s="13">
@@ -1100,7 +1103,7 @@
           <t>Monthly essential expenses</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n"/>
+      <c r="B16" s="19" t="n"/>
       <c r="E16" s="13">
         <f>INDEX(Snapshots!$C$4:$Z$4,10)</f>
         <v/>
@@ -1116,7 +1119,7 @@
           <t>Cash on hand</t>
         </is>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="20">
         <f>IFERROR(INDEX(Snapshots!$C$52:$Z$52,MATCH(2,Snapshots!$C$53:$Z$53)),"")</f>
         <v/>
       </c>
@@ -1135,7 +1138,7 @@
           <t>Months of expenses covered</t>
         </is>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="21">
         <f>IF(AND(ISNUMBER(B16),B16&gt;0,ISNUMBER(B17)),B17/B16,"")</f>
         <v/>
       </c>
@@ -1219,7 +1222,7 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A23),"")</f>
         <v/>
       </c>
@@ -1242,7 +1245,7 @@
           <t>Taxable investing</t>
         </is>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A24),"")</f>
         <v/>
       </c>
@@ -1265,7 +1268,7 @@
           <t>Retirement</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A25),"")</f>
         <v/>
       </c>
@@ -1288,7 +1291,7 @@
           <t>HSA</t>
         </is>
       </c>
-      <c r="B26" s="19">
+      <c r="B26" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A26),"")</f>
         <v/>
       </c>
@@ -1311,7 +1314,7 @@
           <t>Real estate</t>
         </is>
       </c>
-      <c r="B27" s="19">
+      <c r="B27" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A27),"")</f>
         <v/>
       </c>
@@ -1334,7 +1337,7 @@
           <t>Vehicle</t>
         </is>
       </c>
-      <c r="B28" s="19">
+      <c r="B28" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A28),"")</f>
         <v/>
       </c>
@@ -1357,7 +1360,7 @@
           <t>Other asset</t>
         </is>
       </c>
-      <c r="B29" s="19">
+      <c r="B29" s="20">
         <f>IFERROR(SUMIFS(INDEX(Snapshots!$C$5:$Z$44,0,MATCH(2,Snapshots!$C$53:$Z$53)),Accounts!$B$5:$B$44,A29),"")</f>
         <v/>
       </c>
@@ -1385,6 +1388,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:C14"/>
+  </mergeCells>
   <conditionalFormatting sqref="F7:F30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>ISERROR(F7)</formula>
@@ -1467,11 +1473,11 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="22">
         <f>IF(B5="","",VLOOKUP(B5,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="22">
         <f>IF(B5="","",IF(VLOOKUP(B5,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1488,11 +1494,11 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <f>IF(B6="","",VLOOKUP(B6,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="22">
         <f>IF(B6="","",IF(VLOOKUP(B6,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1509,11 +1515,11 @@
           <t>Taxable investing</t>
         </is>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <f>IF(B7="","",VLOOKUP(B7,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="22">
         <f>IF(B7="","",IF(VLOOKUP(B7,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1530,11 +1536,11 @@
           <t>Retirement</t>
         </is>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <f>IF(B8="","",VLOOKUP(B8,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D8" s="21">
+      <c r="D8" s="22">
         <f>IF(B8="","",IF(VLOOKUP(B8,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1551,11 +1557,11 @@
           <t>Retirement</t>
         </is>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <f>IF(B9="","",VLOOKUP(B9,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="22">
         <f>IF(B9="","",IF(VLOOKUP(B9,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1572,11 +1578,11 @@
           <t>HSA</t>
         </is>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="22">
         <f>IF(B10="","",VLOOKUP(B10,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D10" s="21">
+      <c r="D10" s="22">
         <f>IF(B10="","",IF(VLOOKUP(B10,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1593,11 +1599,11 @@
           <t>Real estate</t>
         </is>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="22">
         <f>IF(B11="","",VLOOKUP(B11,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D11" s="21">
+      <c r="D11" s="22">
         <f>IF(B11="","",IF(VLOOKUP(B11,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1614,11 +1620,11 @@
           <t>Vehicle</t>
         </is>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="22">
         <f>IF(B12="","",VLOOKUP(B12,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D12" s="21">
+      <c r="D12" s="22">
         <f>IF(B12="","",IF(VLOOKUP(B12,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1635,11 +1641,11 @@
           <t>Mortgage</t>
         </is>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="22">
         <f>IF(B13="","",VLOOKUP(B13,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D13" s="21">
+      <c r="D13" s="22">
         <f>IF(B13="","",IF(VLOOKUP(B13,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1656,11 +1662,11 @@
           <t>Auto loan</t>
         </is>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="22">
         <f>IF(B14="","",VLOOKUP(B14,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D14" s="21">
+      <c r="D14" s="22">
         <f>IF(B14="","",IF(VLOOKUP(B14,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1677,11 +1683,11 @@
           <t>Student loan</t>
         </is>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="22">
         <f>IF(B15="","",VLOOKUP(B15,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="22">
         <f>IF(B15="","",IF(VLOOKUP(B15,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1698,11 +1704,11 @@
           <t>Credit card</t>
         </is>
       </c>
-      <c r="C16" s="21">
+      <c r="C16" s="22">
         <f>IF(B16="","",VLOOKUP(B16,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D16" s="21">
+      <c r="D16" s="22">
         <f>IF(B16="","",IF(VLOOKUP(B16,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1711,11 +1717,11 @@
     <row r="17">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="21">
+      <c r="C17" s="22">
         <f>IF(B17="","",VLOOKUP(B17,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D17" s="21">
+      <c r="D17" s="22">
         <f>IF(B17="","",IF(VLOOKUP(B17,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1724,11 +1730,11 @@
     <row r="18">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6" t="n"/>
-      <c r="C18" s="21">
+      <c r="C18" s="22">
         <f>IF(B18="","",VLOOKUP(B18,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D18" s="21">
+      <c r="D18" s="22">
         <f>IF(B18="","",IF(VLOOKUP(B18,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1737,11 +1743,11 @@
     <row r="19">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="n"/>
-      <c r="C19" s="21">
+      <c r="C19" s="22">
         <f>IF(B19="","",VLOOKUP(B19,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="22">
         <f>IF(B19="","",IF(VLOOKUP(B19,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1750,11 +1756,11 @@
     <row r="20">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="n"/>
-      <c r="C20" s="21">
+      <c r="C20" s="22">
         <f>IF(B20="","",VLOOKUP(B20,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D20" s="21">
+      <c r="D20" s="22">
         <f>IF(B20="","",IF(VLOOKUP(B20,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1763,11 +1769,11 @@
     <row r="21">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6" t="n"/>
-      <c r="C21" s="21">
+      <c r="C21" s="22">
         <f>IF(B21="","",VLOOKUP(B21,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="22">
         <f>IF(B21="","",IF(VLOOKUP(B21,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1776,11 +1782,11 @@
     <row r="22">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="6" t="n"/>
-      <c r="C22" s="21">
+      <c r="C22" s="22">
         <f>IF(B22="","",VLOOKUP(B22,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="22">
         <f>IF(B22="","",IF(VLOOKUP(B22,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1789,11 +1795,11 @@
     <row r="23">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="n"/>
-      <c r="C23" s="21">
+      <c r="C23" s="22">
         <f>IF(B23="","",VLOOKUP(B23,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="22">
         <f>IF(B23="","",IF(VLOOKUP(B23,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1802,11 +1808,11 @@
     <row r="24">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6" t="n"/>
-      <c r="C24" s="21">
+      <c r="C24" s="22">
         <f>IF(B24="","",VLOOKUP(B24,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D24" s="21">
+      <c r="D24" s="22">
         <f>IF(B24="","",IF(VLOOKUP(B24,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1815,11 +1821,11 @@
     <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="n"/>
-      <c r="C25" s="21">
+      <c r="C25" s="22">
         <f>IF(B25="","",VLOOKUP(B25,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D25" s="21">
+      <c r="D25" s="22">
         <f>IF(B25="","",IF(VLOOKUP(B25,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1828,11 +1834,11 @@
     <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="n"/>
-      <c r="C26" s="21">
+      <c r="C26" s="22">
         <f>IF(B26="","",VLOOKUP(B26,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D26" s="21">
+      <c r="D26" s="22">
         <f>IF(B26="","",IF(VLOOKUP(B26,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1841,11 +1847,11 @@
     <row r="27">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="6" t="n"/>
-      <c r="C27" s="21">
+      <c r="C27" s="22">
         <f>IF(B27="","",VLOOKUP(B27,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D27" s="21">
+      <c r="D27" s="22">
         <f>IF(B27="","",IF(VLOOKUP(B27,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1854,11 +1860,11 @@
     <row r="28">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="6" t="n"/>
-      <c r="C28" s="21">
+      <c r="C28" s="22">
         <f>IF(B28="","",VLOOKUP(B28,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D28" s="21">
+      <c r="D28" s="22">
         <f>IF(B28="","",IF(VLOOKUP(B28,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1867,11 +1873,11 @@
     <row r="29">
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="n"/>
-      <c r="C29" s="21">
+      <c r="C29" s="22">
         <f>IF(B29="","",VLOOKUP(B29,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D29" s="21">
+      <c r="D29" s="22">
         <f>IF(B29="","",IF(VLOOKUP(B29,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1880,11 +1886,11 @@
     <row r="30">
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="6" t="n"/>
-      <c r="C30" s="21">
+      <c r="C30" s="22">
         <f>IF(B30="","",VLOOKUP(B30,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D30" s="21">
+      <c r="D30" s="22">
         <f>IF(B30="","",IF(VLOOKUP(B30,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1893,11 +1899,11 @@
     <row r="31">
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="n"/>
-      <c r="C31" s="21">
+      <c r="C31" s="22">
         <f>IF(B31="","",VLOOKUP(B31,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D31" s="21">
+      <c r="D31" s="22">
         <f>IF(B31="","",IF(VLOOKUP(B31,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1906,11 +1912,11 @@
     <row r="32">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="n"/>
-      <c r="C32" s="21">
+      <c r="C32" s="22">
         <f>IF(B32="","",VLOOKUP(B32,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D32" s="21">
+      <c r="D32" s="22">
         <f>IF(B32="","",IF(VLOOKUP(B32,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1919,11 +1925,11 @@
     <row r="33">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="n"/>
-      <c r="C33" s="21">
+      <c r="C33" s="22">
         <f>IF(B33="","",VLOOKUP(B33,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="22">
         <f>IF(B33="","",IF(VLOOKUP(B33,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1932,11 +1938,11 @@
     <row r="34">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="n"/>
-      <c r="C34" s="21">
+      <c r="C34" s="22">
         <f>IF(B34="","",VLOOKUP(B34,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="22">
         <f>IF(B34="","",IF(VLOOKUP(B34,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1945,11 +1951,11 @@
     <row r="35">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="n"/>
-      <c r="C35" s="21">
+      <c r="C35" s="22">
         <f>IF(B35="","",VLOOKUP(B35,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="22">
         <f>IF(B35="","",IF(VLOOKUP(B35,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1958,11 +1964,11 @@
     <row r="36">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6" t="n"/>
-      <c r="C36" s="21">
+      <c r="C36" s="22">
         <f>IF(B36="","",VLOOKUP(B36,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="22">
         <f>IF(B36="","",IF(VLOOKUP(B36,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1971,11 +1977,11 @@
     <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="n"/>
-      <c r="C37" s="21">
+      <c r="C37" s="22">
         <f>IF(B37="","",VLOOKUP(B37,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="22">
         <f>IF(B37="","",IF(VLOOKUP(B37,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1984,11 +1990,11 @@
     <row r="38">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6" t="n"/>
-      <c r="C38" s="21">
+      <c r="C38" s="22">
         <f>IF(B38="","",VLOOKUP(B38,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="22">
         <f>IF(B38="","",IF(VLOOKUP(B38,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -1997,11 +2003,11 @@
     <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="n"/>
-      <c r="C39" s="21">
+      <c r="C39" s="22">
         <f>IF(B39="","",VLOOKUP(B39,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="22">
         <f>IF(B39="","",IF(VLOOKUP(B39,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2010,11 +2016,11 @@
     <row r="40">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="6" t="n"/>
-      <c r="C40" s="21">
+      <c r="C40" s="22">
         <f>IF(B40="","",VLOOKUP(B40,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="22">
         <f>IF(B40="","",IF(VLOOKUP(B40,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2023,11 +2029,11 @@
     <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6" t="n"/>
-      <c r="C41" s="21">
+      <c r="C41" s="22">
         <f>IF(B41="","",VLOOKUP(B41,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D41" s="21">
+      <c r="D41" s="22">
         <f>IF(B41="","",IF(VLOOKUP(B41,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2036,11 +2042,11 @@
     <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="6" t="n"/>
-      <c r="C42" s="21">
+      <c r="C42" s="22">
         <f>IF(B42="","",VLOOKUP(B42,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D42" s="21">
+      <c r="D42" s="22">
         <f>IF(B42="","",IF(VLOOKUP(B42,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2049,11 +2055,11 @@
     <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6" t="n"/>
-      <c r="C43" s="21">
+      <c r="C43" s="22">
         <f>IF(B43="","",VLOOKUP(B43,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="22">
         <f>IF(B43="","",IF(VLOOKUP(B43,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2062,11 +2068,11 @@
     <row r="44">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="6" t="n"/>
-      <c r="C44" s="21">
+      <c r="C44" s="22">
         <f>IF(B44="","",VLOOKUP(B44,Lists!$A$5:$C$16,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D44" s="21">
+      <c r="D44" s="22">
         <f>IF(B44="","",IF(VLOOKUP(B44,Lists!$A$5:$C$16,3,FALSE)="Yes","Yes",""))</f>
         <v/>
       </c>
@@ -2152,98 +2158,98 @@
           <t>Type</t>
         </is>
       </c>
-      <c r="C4" s="22" t="n">
+      <c r="C4" s="23" t="n">
         <v>46023</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="24">
         <f>EDATE(C4,1)</f>
         <v/>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="24">
         <f>EDATE(D4,1)</f>
         <v/>
       </c>
-      <c r="F4" s="23">
+      <c r="F4" s="24">
         <f>EDATE(E4,1)</f>
         <v/>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="24">
         <f>EDATE(F4,1)</f>
         <v/>
       </c>
-      <c r="H4" s="23">
+      <c r="H4" s="24">
         <f>EDATE(G4,1)</f>
         <v/>
       </c>
-      <c r="I4" s="23">
+      <c r="I4" s="24">
         <f>EDATE(H4,1)</f>
         <v/>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="24">
         <f>EDATE(I4,1)</f>
         <v/>
       </c>
-      <c r="K4" s="23">
+      <c r="K4" s="24">
         <f>EDATE(J4,1)</f>
         <v/>
       </c>
-      <c r="L4" s="23">
+      <c r="L4" s="24">
         <f>EDATE(K4,1)</f>
         <v/>
       </c>
-      <c r="M4" s="23">
+      <c r="M4" s="24">
         <f>EDATE(L4,1)</f>
         <v/>
       </c>
-      <c r="N4" s="23">
+      <c r="N4" s="24">
         <f>EDATE(M4,1)</f>
         <v/>
       </c>
-      <c r="O4" s="23">
+      <c r="O4" s="24">
         <f>EDATE(N4,1)</f>
         <v/>
       </c>
-      <c r="P4" s="23">
+      <c r="P4" s="24">
         <f>EDATE(O4,1)</f>
         <v/>
       </c>
-      <c r="Q4" s="23">
+      <c r="Q4" s="24">
         <f>EDATE(P4,1)</f>
         <v/>
       </c>
-      <c r="R4" s="23">
+      <c r="R4" s="24">
         <f>EDATE(Q4,1)</f>
         <v/>
       </c>
-      <c r="S4" s="23">
+      <c r="S4" s="24">
         <f>EDATE(R4,1)</f>
         <v/>
       </c>
-      <c r="T4" s="23">
+      <c r="T4" s="24">
         <f>EDATE(S4,1)</f>
         <v/>
       </c>
-      <c r="U4" s="23">
+      <c r="U4" s="24">
         <f>EDATE(T4,1)</f>
         <v/>
       </c>
-      <c r="V4" s="23">
+      <c r="V4" s="24">
         <f>EDATE(U4,1)</f>
         <v/>
       </c>
-      <c r="W4" s="23">
+      <c r="W4" s="24">
         <f>EDATE(V4,1)</f>
         <v/>
       </c>
-      <c r="X4" s="23">
+      <c r="X4" s="24">
         <f>EDATE(W4,1)</f>
         <v/>
       </c>
-      <c r="Y4" s="23">
+      <c r="Y4" s="24">
         <f>EDATE(X4,1)</f>
         <v/>
       </c>
-      <c r="Z4" s="23">
+      <c r="Z4" s="24">
         <f>EDATE(Y4,1)</f>
         <v/>
       </c>
@@ -2253,1360 +2259,1360 @@
         <f>IF(Accounts!A5="","",Accounts!A5)</f>
         <v/>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="22">
         <f>IF(Accounts!B5="","",Accounts!B5)</f>
         <v/>
       </c>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
-      <c r="E5" s="18" t="n"/>
-      <c r="F5" s="18" t="n"/>
-      <c r="G5" s="18" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="18" t="n"/>
-      <c r="J5" s="18" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="18" t="n"/>
-      <c r="M5" s="18" t="n"/>
-      <c r="N5" s="18" t="n"/>
-      <c r="O5" s="18" t="n"/>
-      <c r="P5" s="18" t="n"/>
-      <c r="Q5" s="18" t="n"/>
-      <c r="R5" s="18" t="n"/>
-      <c r="S5" s="18" t="n"/>
-      <c r="T5" s="18" t="n"/>
-      <c r="U5" s="18" t="n"/>
-      <c r="V5" s="18" t="n"/>
-      <c r="W5" s="18" t="n"/>
-      <c r="X5" s="18" t="n"/>
-      <c r="Y5" s="18" t="n"/>
-      <c r="Z5" s="18" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="19" t="n"/>
+      <c r="H5" s="19" t="n"/>
+      <c r="I5" s="19" t="n"/>
+      <c r="J5" s="19" t="n"/>
+      <c r="K5" s="19" t="n"/>
+      <c r="L5" s="19" t="n"/>
+      <c r="M5" s="19" t="n"/>
+      <c r="N5" s="19" t="n"/>
+      <c r="O5" s="19" t="n"/>
+      <c r="P5" s="19" t="n"/>
+      <c r="Q5" s="19" t="n"/>
+      <c r="R5" s="19" t="n"/>
+      <c r="S5" s="19" t="n"/>
+      <c r="T5" s="19" t="n"/>
+      <c r="U5" s="19" t="n"/>
+      <c r="V5" s="19" t="n"/>
+      <c r="W5" s="19" t="n"/>
+      <c r="X5" s="19" t="n"/>
+      <c r="Y5" s="19" t="n"/>
+      <c r="Z5" s="19" t="n"/>
     </row>
     <row r="6">
       <c r="A6">
         <f>IF(Accounts!A6="","",Accounts!A6)</f>
         <v/>
       </c>
-      <c r="B6" s="21">
+      <c r="B6" s="22">
         <f>IF(Accounts!B6="","",Accounts!B6)</f>
         <v/>
       </c>
-      <c r="C6" s="18" t="n"/>
-      <c r="D6" s="18" t="n"/>
-      <c r="E6" s="18" t="n"/>
-      <c r="F6" s="18" t="n"/>
-      <c r="G6" s="18" t="n"/>
-      <c r="H6" s="18" t="n"/>
-      <c r="I6" s="18" t="n"/>
-      <c r="J6" s="18" t="n"/>
-      <c r="K6" s="18" t="n"/>
-      <c r="L6" s="18" t="n"/>
-      <c r="M6" s="18" t="n"/>
-      <c r="N6" s="18" t="n"/>
-      <c r="O6" s="18" t="n"/>
-      <c r="P6" s="18" t="n"/>
-      <c r="Q6" s="18" t="n"/>
-      <c r="R6" s="18" t="n"/>
-      <c r="S6" s="18" t="n"/>
-      <c r="T6" s="18" t="n"/>
-      <c r="U6" s="18" t="n"/>
-      <c r="V6" s="18" t="n"/>
-      <c r="W6" s="18" t="n"/>
-      <c r="X6" s="18" t="n"/>
-      <c r="Y6" s="18" t="n"/>
-      <c r="Z6" s="18" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="19" t="n"/>
+      <c r="I6" s="19" t="n"/>
+      <c r="J6" s="19" t="n"/>
+      <c r="K6" s="19" t="n"/>
+      <c r="L6" s="19" t="n"/>
+      <c r="M6" s="19" t="n"/>
+      <c r="N6" s="19" t="n"/>
+      <c r="O6" s="19" t="n"/>
+      <c r="P6" s="19" t="n"/>
+      <c r="Q6" s="19" t="n"/>
+      <c r="R6" s="19" t="n"/>
+      <c r="S6" s="19" t="n"/>
+      <c r="T6" s="19" t="n"/>
+      <c r="U6" s="19" t="n"/>
+      <c r="V6" s="19" t="n"/>
+      <c r="W6" s="19" t="n"/>
+      <c r="X6" s="19" t="n"/>
+      <c r="Y6" s="19" t="n"/>
+      <c r="Z6" s="19" t="n"/>
     </row>
     <row r="7">
       <c r="A7">
         <f>IF(Accounts!A7="","",Accounts!A7)</f>
         <v/>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="22">
         <f>IF(Accounts!B7="","",Accounts!B7)</f>
         <v/>
       </c>
-      <c r="C7" s="18" t="n"/>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="18" t="n"/>
-      <c r="N7" s="18" t="n"/>
-      <c r="O7" s="18" t="n"/>
-      <c r="P7" s="18" t="n"/>
-      <c r="Q7" s="18" t="n"/>
-      <c r="R7" s="18" t="n"/>
-      <c r="S7" s="18" t="n"/>
-      <c r="T7" s="18" t="n"/>
-      <c r="U7" s="18" t="n"/>
-      <c r="V7" s="18" t="n"/>
-      <c r="W7" s="18" t="n"/>
-      <c r="X7" s="18" t="n"/>
-      <c r="Y7" s="18" t="n"/>
-      <c r="Z7" s="18" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="19" t="n"/>
+      <c r="K7" s="19" t="n"/>
+      <c r="L7" s="19" t="n"/>
+      <c r="M7" s="19" t="n"/>
+      <c r="N7" s="19" t="n"/>
+      <c r="O7" s="19" t="n"/>
+      <c r="P7" s="19" t="n"/>
+      <c r="Q7" s="19" t="n"/>
+      <c r="R7" s="19" t="n"/>
+      <c r="S7" s="19" t="n"/>
+      <c r="T7" s="19" t="n"/>
+      <c r="U7" s="19" t="n"/>
+      <c r="V7" s="19" t="n"/>
+      <c r="W7" s="19" t="n"/>
+      <c r="X7" s="19" t="n"/>
+      <c r="Y7" s="19" t="n"/>
+      <c r="Z7" s="19" t="n"/>
     </row>
     <row r="8">
       <c r="A8">
         <f>IF(Accounts!A8="","",Accounts!A8)</f>
         <v/>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="22">
         <f>IF(Accounts!B8="","",Accounts!B8)</f>
         <v/>
       </c>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="18" t="n"/>
-      <c r="N8" s="18" t="n"/>
-      <c r="O8" s="18" t="n"/>
-      <c r="P8" s="18" t="n"/>
-      <c r="Q8" s="18" t="n"/>
-      <c r="R8" s="18" t="n"/>
-      <c r="S8" s="18" t="n"/>
-      <c r="T8" s="18" t="n"/>
-      <c r="U8" s="18" t="n"/>
-      <c r="V8" s="18" t="n"/>
-      <c r="W8" s="18" t="n"/>
-      <c r="X8" s="18" t="n"/>
-      <c r="Y8" s="18" t="n"/>
-      <c r="Z8" s="18" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="19" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="19" t="n"/>
+      <c r="P8" s="19" t="n"/>
+      <c r="Q8" s="19" t="n"/>
+      <c r="R8" s="19" t="n"/>
+      <c r="S8" s="19" t="n"/>
+      <c r="T8" s="19" t="n"/>
+      <c r="U8" s="19" t="n"/>
+      <c r="V8" s="19" t="n"/>
+      <c r="W8" s="19" t="n"/>
+      <c r="X8" s="19" t="n"/>
+      <c r="Y8" s="19" t="n"/>
+      <c r="Z8" s="19" t="n"/>
     </row>
     <row r="9">
       <c r="A9">
         <f>IF(Accounts!A9="","",Accounts!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="22">
         <f>IF(Accounts!B9="","",Accounts!B9)</f>
         <v/>
       </c>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="18" t="n"/>
-      <c r="K9" s="18" t="n"/>
-      <c r="L9" s="18" t="n"/>
-      <c r="M9" s="18" t="n"/>
-      <c r="N9" s="18" t="n"/>
-      <c r="O9" s="18" t="n"/>
-      <c r="P9" s="18" t="n"/>
-      <c r="Q9" s="18" t="n"/>
-      <c r="R9" s="18" t="n"/>
-      <c r="S9" s="18" t="n"/>
-      <c r="T9" s="18" t="n"/>
-      <c r="U9" s="18" t="n"/>
-      <c r="V9" s="18" t="n"/>
-      <c r="W9" s="18" t="n"/>
-      <c r="X9" s="18" t="n"/>
-      <c r="Y9" s="18" t="n"/>
-      <c r="Z9" s="18" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="19" t="n"/>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="19" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="19" t="n"/>
+      <c r="O9" s="19" t="n"/>
+      <c r="P9" s="19" t="n"/>
+      <c r="Q9" s="19" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
+      <c r="T9" s="19" t="n"/>
+      <c r="U9" s="19" t="n"/>
+      <c r="V9" s="19" t="n"/>
+      <c r="W9" s="19" t="n"/>
+      <c r="X9" s="19" t="n"/>
+      <c r="Y9" s="19" t="n"/>
+      <c r="Z9" s="19" t="n"/>
     </row>
     <row r="10">
       <c r="A10">
         <f>IF(Accounts!A10="","",Accounts!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="22">
         <f>IF(Accounts!B10="","",Accounts!B10)</f>
         <v/>
       </c>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="18" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="18" t="n"/>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="18" t="n"/>
-      <c r="K10" s="18" t="n"/>
-      <c r="L10" s="18" t="n"/>
-      <c r="M10" s="18" t="n"/>
-      <c r="N10" s="18" t="n"/>
-      <c r="O10" s="18" t="n"/>
-      <c r="P10" s="18" t="n"/>
-      <c r="Q10" s="18" t="n"/>
-      <c r="R10" s="18" t="n"/>
-      <c r="S10" s="18" t="n"/>
-      <c r="T10" s="18" t="n"/>
-      <c r="U10" s="18" t="n"/>
-      <c r="V10" s="18" t="n"/>
-      <c r="W10" s="18" t="n"/>
-      <c r="X10" s="18" t="n"/>
-      <c r="Y10" s="18" t="n"/>
-      <c r="Z10" s="18" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="19" t="n"/>
+      <c r="N10" s="19" t="n"/>
+      <c r="O10" s="19" t="n"/>
+      <c r="P10" s="19" t="n"/>
+      <c r="Q10" s="19" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
+      <c r="T10" s="19" t="n"/>
+      <c r="U10" s="19" t="n"/>
+      <c r="V10" s="19" t="n"/>
+      <c r="W10" s="19" t="n"/>
+      <c r="X10" s="19" t="n"/>
+      <c r="Y10" s="19" t="n"/>
+      <c r="Z10" s="19" t="n"/>
     </row>
     <row r="11">
       <c r="A11">
         <f>IF(Accounts!A11="","",Accounts!A11)</f>
         <v/>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="22">
         <f>IF(Accounts!B11="","",Accounts!B11)</f>
         <v/>
       </c>
-      <c r="C11" s="18" t="n"/>
-      <c r="D11" s="18" t="n"/>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="18" t="n"/>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="18" t="n"/>
-      <c r="L11" s="18" t="n"/>
-      <c r="M11" s="18" t="n"/>
-      <c r="N11" s="18" t="n"/>
-      <c r="O11" s="18" t="n"/>
-      <c r="P11" s="18" t="n"/>
-      <c r="Q11" s="18" t="n"/>
-      <c r="R11" s="18" t="n"/>
-      <c r="S11" s="18" t="n"/>
-      <c r="T11" s="18" t="n"/>
-      <c r="U11" s="18" t="n"/>
-      <c r="V11" s="18" t="n"/>
-      <c r="W11" s="18" t="n"/>
-      <c r="X11" s="18" t="n"/>
-      <c r="Y11" s="18" t="n"/>
-      <c r="Z11" s="18" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="19" t="n"/>
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
+      <c r="M11" s="19" t="n"/>
+      <c r="N11" s="19" t="n"/>
+      <c r="O11" s="19" t="n"/>
+      <c r="P11" s="19" t="n"/>
+      <c r="Q11" s="19" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
+      <c r="T11" s="19" t="n"/>
+      <c r="U11" s="19" t="n"/>
+      <c r="V11" s="19" t="n"/>
+      <c r="W11" s="19" t="n"/>
+      <c r="X11" s="19" t="n"/>
+      <c r="Y11" s="19" t="n"/>
+      <c r="Z11" s="19" t="n"/>
     </row>
     <row r="12">
       <c r="A12">
         <f>IF(Accounts!A12="","",Accounts!A12)</f>
         <v/>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="22">
         <f>IF(Accounts!B12="","",Accounts!B12)</f>
         <v/>
       </c>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="18" t="n"/>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="18" t="n"/>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="18" t="n"/>
-      <c r="K12" s="18" t="n"/>
-      <c r="L12" s="18" t="n"/>
-      <c r="M12" s="18" t="n"/>
-      <c r="N12" s="18" t="n"/>
-      <c r="O12" s="18" t="n"/>
-      <c r="P12" s="18" t="n"/>
-      <c r="Q12" s="18" t="n"/>
-      <c r="R12" s="18" t="n"/>
-      <c r="S12" s="18" t="n"/>
-      <c r="T12" s="18" t="n"/>
-      <c r="U12" s="18" t="n"/>
-      <c r="V12" s="18" t="n"/>
-      <c r="W12" s="18" t="n"/>
-      <c r="X12" s="18" t="n"/>
-      <c r="Y12" s="18" t="n"/>
-      <c r="Z12" s="18" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+      <c r="H12" s="19" t="n"/>
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="19" t="n"/>
+      <c r="O12" s="19" t="n"/>
+      <c r="P12" s="19" t="n"/>
+      <c r="Q12" s="19" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
+      <c r="T12" s="19" t="n"/>
+      <c r="U12" s="19" t="n"/>
+      <c r="V12" s="19" t="n"/>
+      <c r="W12" s="19" t="n"/>
+      <c r="X12" s="19" t="n"/>
+      <c r="Y12" s="19" t="n"/>
+      <c r="Z12" s="19" t="n"/>
     </row>
     <row r="13">
       <c r="A13">
         <f>IF(Accounts!A13="","",Accounts!A13)</f>
         <v/>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="22">
         <f>IF(Accounts!B13="","",Accounts!B13)</f>
         <v/>
       </c>
-      <c r="C13" s="18" t="n"/>
-      <c r="D13" s="18" t="n"/>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="18" t="n"/>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="18" t="n"/>
-      <c r="J13" s="18" t="n"/>
-      <c r="K13" s="18" t="n"/>
-      <c r="L13" s="18" t="n"/>
-      <c r="M13" s="18" t="n"/>
-      <c r="N13" s="18" t="n"/>
-      <c r="O13" s="18" t="n"/>
-      <c r="P13" s="18" t="n"/>
-      <c r="Q13" s="18" t="n"/>
-      <c r="R13" s="18" t="n"/>
-      <c r="S13" s="18" t="n"/>
-      <c r="T13" s="18" t="n"/>
-      <c r="U13" s="18" t="n"/>
-      <c r="V13" s="18" t="n"/>
-      <c r="W13" s="18" t="n"/>
-      <c r="X13" s="18" t="n"/>
-      <c r="Y13" s="18" t="n"/>
-      <c r="Z13" s="18" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="19" t="n"/>
+      <c r="L13" s="19" t="n"/>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="19" t="n"/>
+      <c r="O13" s="19" t="n"/>
+      <c r="P13" s="19" t="n"/>
+      <c r="Q13" s="19" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
+      <c r="T13" s="19" t="n"/>
+      <c r="U13" s="19" t="n"/>
+      <c r="V13" s="19" t="n"/>
+      <c r="W13" s="19" t="n"/>
+      <c r="X13" s="19" t="n"/>
+      <c r="Y13" s="19" t="n"/>
+      <c r="Z13" s="19" t="n"/>
     </row>
     <row r="14">
       <c r="A14">
         <f>IF(Accounts!A14="","",Accounts!A14)</f>
         <v/>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="22">
         <f>IF(Accounts!B14="","",Accounts!B14)</f>
         <v/>
       </c>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="18" t="n"/>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="18" t="n"/>
-      <c r="J14" s="18" t="n"/>
-      <c r="K14" s="18" t="n"/>
-      <c r="L14" s="18" t="n"/>
-      <c r="M14" s="18" t="n"/>
-      <c r="N14" s="18" t="n"/>
-      <c r="O14" s="18" t="n"/>
-      <c r="P14" s="18" t="n"/>
-      <c r="Q14" s="18" t="n"/>
-      <c r="R14" s="18" t="n"/>
-      <c r="S14" s="18" t="n"/>
-      <c r="T14" s="18" t="n"/>
-      <c r="U14" s="18" t="n"/>
-      <c r="V14" s="18" t="n"/>
-      <c r="W14" s="18" t="n"/>
-      <c r="X14" s="18" t="n"/>
-      <c r="Y14" s="18" t="n"/>
-      <c r="Z14" s="18" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="19" t="n"/>
+      <c r="N14" s="19" t="n"/>
+      <c r="O14" s="19" t="n"/>
+      <c r="P14" s="19" t="n"/>
+      <c r="Q14" s="19" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
+      <c r="T14" s="19" t="n"/>
+      <c r="U14" s="19" t="n"/>
+      <c r="V14" s="19" t="n"/>
+      <c r="W14" s="19" t="n"/>
+      <c r="X14" s="19" t="n"/>
+      <c r="Y14" s="19" t="n"/>
+      <c r="Z14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15">
         <f>IF(Accounts!A15="","",Accounts!A15)</f>
         <v/>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="22">
         <f>IF(Accounts!B15="","",Accounts!B15)</f>
         <v/>
       </c>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="18" t="n"/>
-      <c r="N15" s="18" t="n"/>
-      <c r="O15" s="18" t="n"/>
-      <c r="P15" s="18" t="n"/>
-      <c r="Q15" s="18" t="n"/>
-      <c r="R15" s="18" t="n"/>
-      <c r="S15" s="18" t="n"/>
-      <c r="T15" s="18" t="n"/>
-      <c r="U15" s="18" t="n"/>
-      <c r="V15" s="18" t="n"/>
-      <c r="W15" s="18" t="n"/>
-      <c r="X15" s="18" t="n"/>
-      <c r="Y15" s="18" t="n"/>
-      <c r="Z15" s="18" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="19" t="n"/>
+      <c r="O15" s="19" t="n"/>
+      <c r="P15" s="19" t="n"/>
+      <c r="Q15" s="19" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
+      <c r="T15" s="19" t="n"/>
+      <c r="U15" s="19" t="n"/>
+      <c r="V15" s="19" t="n"/>
+      <c r="W15" s="19" t="n"/>
+      <c r="X15" s="19" t="n"/>
+      <c r="Y15" s="19" t="n"/>
+      <c r="Z15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16">
         <f>IF(Accounts!A16="","",Accounts!A16)</f>
         <v/>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="22">
         <f>IF(Accounts!B16="","",Accounts!B16)</f>
         <v/>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
-      <c r="I16" s="18" t="n"/>
-      <c r="J16" s="18" t="n"/>
-      <c r="K16" s="18" t="n"/>
-      <c r="L16" s="18" t="n"/>
-      <c r="M16" s="18" t="n"/>
-      <c r="N16" s="18" t="n"/>
-      <c r="O16" s="18" t="n"/>
-      <c r="P16" s="18" t="n"/>
-      <c r="Q16" s="18" t="n"/>
-      <c r="R16" s="18" t="n"/>
-      <c r="S16" s="18" t="n"/>
-      <c r="T16" s="18" t="n"/>
-      <c r="U16" s="18" t="n"/>
-      <c r="V16" s="18" t="n"/>
-      <c r="W16" s="18" t="n"/>
-      <c r="X16" s="18" t="n"/>
-      <c r="Y16" s="18" t="n"/>
-      <c r="Z16" s="18" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="19" t="n"/>
+      <c r="J16" s="19" t="n"/>
+      <c r="K16" s="19" t="n"/>
+      <c r="L16" s="19" t="n"/>
+      <c r="M16" s="19" t="n"/>
+      <c r="N16" s="19" t="n"/>
+      <c r="O16" s="19" t="n"/>
+      <c r="P16" s="19" t="n"/>
+      <c r="Q16" s="19" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
+      <c r="T16" s="19" t="n"/>
+      <c r="U16" s="19" t="n"/>
+      <c r="V16" s="19" t="n"/>
+      <c r="W16" s="19" t="n"/>
+      <c r="X16" s="19" t="n"/>
+      <c r="Y16" s="19" t="n"/>
+      <c r="Z16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17">
         <f>IF(Accounts!A17="","",Accounts!A17)</f>
         <v/>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="22">
         <f>IF(Accounts!B17="","",Accounts!B17)</f>
         <v/>
       </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="18" t="n"/>
-      <c r="I17" s="18" t="n"/>
-      <c r="J17" s="18" t="n"/>
-      <c r="K17" s="18" t="n"/>
-      <c r="L17" s="18" t="n"/>
-      <c r="M17" s="18" t="n"/>
-      <c r="N17" s="18" t="n"/>
-      <c r="O17" s="18" t="n"/>
-      <c r="P17" s="18" t="n"/>
-      <c r="Q17" s="18" t="n"/>
-      <c r="R17" s="18" t="n"/>
-      <c r="S17" s="18" t="n"/>
-      <c r="T17" s="18" t="n"/>
-      <c r="U17" s="18" t="n"/>
-      <c r="V17" s="18" t="n"/>
-      <c r="W17" s="18" t="n"/>
-      <c r="X17" s="18" t="n"/>
-      <c r="Y17" s="18" t="n"/>
-      <c r="Z17" s="18" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="19" t="n"/>
+      <c r="J17" s="19" t="n"/>
+      <c r="K17" s="19" t="n"/>
+      <c r="L17" s="19" t="n"/>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="19" t="n"/>
+      <c r="O17" s="19" t="n"/>
+      <c r="P17" s="19" t="n"/>
+      <c r="Q17" s="19" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
+      <c r="T17" s="19" t="n"/>
+      <c r="U17" s="19" t="n"/>
+      <c r="V17" s="19" t="n"/>
+      <c r="W17" s="19" t="n"/>
+      <c r="X17" s="19" t="n"/>
+      <c r="Y17" s="19" t="n"/>
+      <c r="Z17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18">
         <f>IF(Accounts!A18="","",Accounts!A18)</f>
         <v/>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="22">
         <f>IF(Accounts!B18="","",Accounts!B18)</f>
         <v/>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
-      <c r="I18" s="18" t="n"/>
-      <c r="J18" s="18" t="n"/>
-      <c r="K18" s="18" t="n"/>
-      <c r="L18" s="18" t="n"/>
-      <c r="M18" s="18" t="n"/>
-      <c r="N18" s="18" t="n"/>
-      <c r="O18" s="18" t="n"/>
-      <c r="P18" s="18" t="n"/>
-      <c r="Q18" s="18" t="n"/>
-      <c r="R18" s="18" t="n"/>
-      <c r="S18" s="18" t="n"/>
-      <c r="T18" s="18" t="n"/>
-      <c r="U18" s="18" t="n"/>
-      <c r="V18" s="18" t="n"/>
-      <c r="W18" s="18" t="n"/>
-      <c r="X18" s="18" t="n"/>
-      <c r="Y18" s="18" t="n"/>
-      <c r="Z18" s="18" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
+      <c r="I18" s="19" t="n"/>
+      <c r="J18" s="19" t="n"/>
+      <c r="K18" s="19" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="19" t="n"/>
+      <c r="O18" s="19" t="n"/>
+      <c r="P18" s="19" t="n"/>
+      <c r="Q18" s="19" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
+      <c r="T18" s="19" t="n"/>
+      <c r="U18" s="19" t="n"/>
+      <c r="V18" s="19" t="n"/>
+      <c r="W18" s="19" t="n"/>
+      <c r="X18" s="19" t="n"/>
+      <c r="Y18" s="19" t="n"/>
+      <c r="Z18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19">
         <f>IF(Accounts!A19="","",Accounts!A19)</f>
         <v/>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="22">
         <f>IF(Accounts!B19="","",Accounts!B19)</f>
         <v/>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
-      <c r="F19" s="18" t="n"/>
-      <c r="G19" s="18" t="n"/>
-      <c r="H19" s="18" t="n"/>
-      <c r="I19" s="18" t="n"/>
-      <c r="J19" s="18" t="n"/>
-      <c r="K19" s="18" t="n"/>
-      <c r="L19" s="18" t="n"/>
-      <c r="M19" s="18" t="n"/>
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="18" t="n"/>
-      <c r="P19" s="18" t="n"/>
-      <c r="Q19" s="18" t="n"/>
-      <c r="R19" s="18" t="n"/>
-      <c r="S19" s="18" t="n"/>
-      <c r="T19" s="18" t="n"/>
-      <c r="U19" s="18" t="n"/>
-      <c r="V19" s="18" t="n"/>
-      <c r="W19" s="18" t="n"/>
-      <c r="X19" s="18" t="n"/>
-      <c r="Y19" s="18" t="n"/>
-      <c r="Z19" s="18" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
+      <c r="H19" s="19" t="n"/>
+      <c r="I19" s="19" t="n"/>
+      <c r="J19" s="19" t="n"/>
+      <c r="K19" s="19" t="n"/>
+      <c r="L19" s="19" t="n"/>
+      <c r="M19" s="19" t="n"/>
+      <c r="N19" s="19" t="n"/>
+      <c r="O19" s="19" t="n"/>
+      <c r="P19" s="19" t="n"/>
+      <c r="Q19" s="19" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
+      <c r="T19" s="19" t="n"/>
+      <c r="U19" s="19" t="n"/>
+      <c r="V19" s="19" t="n"/>
+      <c r="W19" s="19" t="n"/>
+      <c r="X19" s="19" t="n"/>
+      <c r="Y19" s="19" t="n"/>
+      <c r="Z19" s="19" t="n"/>
     </row>
     <row r="20">
       <c r="A20">
         <f>IF(Accounts!A20="","",Accounts!A20)</f>
         <v/>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="22">
         <f>IF(Accounts!B20="","",Accounts!B20)</f>
         <v/>
       </c>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="18" t="n"/>
-      <c r="I20" s="18" t="n"/>
-      <c r="J20" s="18" t="n"/>
-      <c r="K20" s="18" t="n"/>
-      <c r="L20" s="18" t="n"/>
-      <c r="M20" s="18" t="n"/>
-      <c r="N20" s="18" t="n"/>
-      <c r="O20" s="18" t="n"/>
-      <c r="P20" s="18" t="n"/>
-      <c r="Q20" s="18" t="n"/>
-      <c r="R20" s="18" t="n"/>
-      <c r="S20" s="18" t="n"/>
-      <c r="T20" s="18" t="n"/>
-      <c r="U20" s="18" t="n"/>
-      <c r="V20" s="18" t="n"/>
-      <c r="W20" s="18" t="n"/>
-      <c r="X20" s="18" t="n"/>
-      <c r="Y20" s="18" t="n"/>
-      <c r="Z20" s="18" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19" t="n"/>
+      <c r="I20" s="19" t="n"/>
+      <c r="J20" s="19" t="n"/>
+      <c r="K20" s="19" t="n"/>
+      <c r="L20" s="19" t="n"/>
+      <c r="M20" s="19" t="n"/>
+      <c r="N20" s="19" t="n"/>
+      <c r="O20" s="19" t="n"/>
+      <c r="P20" s="19" t="n"/>
+      <c r="Q20" s="19" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
+      <c r="T20" s="19" t="n"/>
+      <c r="U20" s="19" t="n"/>
+      <c r="V20" s="19" t="n"/>
+      <c r="W20" s="19" t="n"/>
+      <c r="X20" s="19" t="n"/>
+      <c r="Y20" s="19" t="n"/>
+      <c r="Z20" s="19" t="n"/>
     </row>
     <row r="21">
       <c r="A21">
         <f>IF(Accounts!A21="","",Accounts!A21)</f>
         <v/>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="22">
         <f>IF(Accounts!B21="","",Accounts!B21)</f>
         <v/>
       </c>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
-      <c r="E21" s="18" t="n"/>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="18" t="n"/>
-      <c r="I21" s="18" t="n"/>
-      <c r="J21" s="18" t="n"/>
-      <c r="K21" s="18" t="n"/>
-      <c r="L21" s="18" t="n"/>
-      <c r="M21" s="18" t="n"/>
-      <c r="N21" s="18" t="n"/>
-      <c r="O21" s="18" t="n"/>
-      <c r="P21" s="18" t="n"/>
-      <c r="Q21" s="18" t="n"/>
-      <c r="R21" s="18" t="n"/>
-      <c r="S21" s="18" t="n"/>
-      <c r="T21" s="18" t="n"/>
-      <c r="U21" s="18" t="n"/>
-      <c r="V21" s="18" t="n"/>
-      <c r="W21" s="18" t="n"/>
-      <c r="X21" s="18" t="n"/>
-      <c r="Y21" s="18" t="n"/>
-      <c r="Z21" s="18" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="19" t="n"/>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="19" t="n"/>
+      <c r="O21" s="19" t="n"/>
+      <c r="P21" s="19" t="n"/>
+      <c r="Q21" s="19" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
+      <c r="T21" s="19" t="n"/>
+      <c r="U21" s="19" t="n"/>
+      <c r="V21" s="19" t="n"/>
+      <c r="W21" s="19" t="n"/>
+      <c r="X21" s="19" t="n"/>
+      <c r="Y21" s="19" t="n"/>
+      <c r="Z21" s="19" t="n"/>
     </row>
     <row r="22">
       <c r="A22">
         <f>IF(Accounts!A22="","",Accounts!A22)</f>
         <v/>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="22">
         <f>IF(Accounts!B22="","",Accounts!B22)</f>
         <v/>
       </c>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
-      <c r="E22" s="18" t="n"/>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="18" t="n"/>
-      <c r="I22" s="18" t="n"/>
-      <c r="J22" s="18" t="n"/>
-      <c r="K22" s="18" t="n"/>
-      <c r="L22" s="18" t="n"/>
-      <c r="M22" s="18" t="n"/>
-      <c r="N22" s="18" t="n"/>
-      <c r="O22" s="18" t="n"/>
-      <c r="P22" s="18" t="n"/>
-      <c r="Q22" s="18" t="n"/>
-      <c r="R22" s="18" t="n"/>
-      <c r="S22" s="18" t="n"/>
-      <c r="T22" s="18" t="n"/>
-      <c r="U22" s="18" t="n"/>
-      <c r="V22" s="18" t="n"/>
-      <c r="W22" s="18" t="n"/>
-      <c r="X22" s="18" t="n"/>
-      <c r="Y22" s="18" t="n"/>
-      <c r="Z22" s="18" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
+      <c r="I22" s="19" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="n"/>
+      <c r="O22" s="19" t="n"/>
+      <c r="P22" s="19" t="n"/>
+      <c r="Q22" s="19" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
+      <c r="T22" s="19" t="n"/>
+      <c r="U22" s="19" t="n"/>
+      <c r="V22" s="19" t="n"/>
+      <c r="W22" s="19" t="n"/>
+      <c r="X22" s="19" t="n"/>
+      <c r="Y22" s="19" t="n"/>
+      <c r="Z22" s="19" t="n"/>
     </row>
     <row r="23">
       <c r="A23">
         <f>IF(Accounts!A23="","",Accounts!A23)</f>
         <v/>
       </c>
-      <c r="B23" s="21">
+      <c r="B23" s="22">
         <f>IF(Accounts!B23="","",Accounts!B23)</f>
         <v/>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="18" t="n"/>
-      <c r="I23" s="18" t="n"/>
-      <c r="J23" s="18" t="n"/>
-      <c r="K23" s="18" t="n"/>
-      <c r="L23" s="18" t="n"/>
-      <c r="M23" s="18" t="n"/>
-      <c r="N23" s="18" t="n"/>
-      <c r="O23" s="18" t="n"/>
-      <c r="P23" s="18" t="n"/>
-      <c r="Q23" s="18" t="n"/>
-      <c r="R23" s="18" t="n"/>
-      <c r="S23" s="18" t="n"/>
-      <c r="T23" s="18" t="n"/>
-      <c r="U23" s="18" t="n"/>
-      <c r="V23" s="18" t="n"/>
-      <c r="W23" s="18" t="n"/>
-      <c r="X23" s="18" t="n"/>
-      <c r="Y23" s="18" t="n"/>
-      <c r="Z23" s="18" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="19" t="n"/>
+      <c r="O23" s="19" t="n"/>
+      <c r="P23" s="19" t="n"/>
+      <c r="Q23" s="19" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
+      <c r="T23" s="19" t="n"/>
+      <c r="U23" s="19" t="n"/>
+      <c r="V23" s="19" t="n"/>
+      <c r="W23" s="19" t="n"/>
+      <c r="X23" s="19" t="n"/>
+      <c r="Y23" s="19" t="n"/>
+      <c r="Z23" s="19" t="n"/>
     </row>
     <row r="24">
       <c r="A24">
         <f>IF(Accounts!A24="","",Accounts!A24)</f>
         <v/>
       </c>
-      <c r="B24" s="21">
+      <c r="B24" s="22">
         <f>IF(Accounts!B24="","",Accounts!B24)</f>
         <v/>
       </c>
-      <c r="C24" s="18" t="n"/>
-      <c r="D24" s="18" t="n"/>
-      <c r="E24" s="18" t="n"/>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="18" t="n"/>
-      <c r="I24" s="18" t="n"/>
-      <c r="J24" s="18" t="n"/>
-      <c r="K24" s="18" t="n"/>
-      <c r="L24" s="18" t="n"/>
-      <c r="M24" s="18" t="n"/>
-      <c r="N24" s="18" t="n"/>
-      <c r="O24" s="18" t="n"/>
-      <c r="P24" s="18" t="n"/>
-      <c r="Q24" s="18" t="n"/>
-      <c r="R24" s="18" t="n"/>
-      <c r="S24" s="18" t="n"/>
-      <c r="T24" s="18" t="n"/>
-      <c r="U24" s="18" t="n"/>
-      <c r="V24" s="18" t="n"/>
-      <c r="W24" s="18" t="n"/>
-      <c r="X24" s="18" t="n"/>
-      <c r="Y24" s="18" t="n"/>
-      <c r="Z24" s="18" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
+      <c r="I24" s="19" t="n"/>
+      <c r="J24" s="19" t="n"/>
+      <c r="K24" s="19" t="n"/>
+      <c r="L24" s="19" t="n"/>
+      <c r="M24" s="19" t="n"/>
+      <c r="N24" s="19" t="n"/>
+      <c r="O24" s="19" t="n"/>
+      <c r="P24" s="19" t="n"/>
+      <c r="Q24" s="19" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
+      <c r="T24" s="19" t="n"/>
+      <c r="U24" s="19" t="n"/>
+      <c r="V24" s="19" t="n"/>
+      <c r="W24" s="19" t="n"/>
+      <c r="X24" s="19" t="n"/>
+      <c r="Y24" s="19" t="n"/>
+      <c r="Z24" s="19" t="n"/>
     </row>
     <row r="25">
       <c r="A25">
         <f>IF(Accounts!A25="","",Accounts!A25)</f>
         <v/>
       </c>
-      <c r="B25" s="21">
+      <c r="B25" s="22">
         <f>IF(Accounts!B25="","",Accounts!B25)</f>
         <v/>
       </c>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18" t="n"/>
-      <c r="K25" s="18" t="n"/>
-      <c r="L25" s="18" t="n"/>
-      <c r="M25" s="18" t="n"/>
-      <c r="N25" s="18" t="n"/>
-      <c r="O25" s="18" t="n"/>
-      <c r="P25" s="18" t="n"/>
-      <c r="Q25" s="18" t="n"/>
-      <c r="R25" s="18" t="n"/>
-      <c r="S25" s="18" t="n"/>
-      <c r="T25" s="18" t="n"/>
-      <c r="U25" s="18" t="n"/>
-      <c r="V25" s="18" t="n"/>
-      <c r="W25" s="18" t="n"/>
-      <c r="X25" s="18" t="n"/>
-      <c r="Y25" s="18" t="n"/>
-      <c r="Z25" s="18" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="19" t="n"/>
+      <c r="K25" s="19" t="n"/>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="19" t="n"/>
+      <c r="O25" s="19" t="n"/>
+      <c r="P25" s="19" t="n"/>
+      <c r="Q25" s="19" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
+      <c r="T25" s="19" t="n"/>
+      <c r="U25" s="19" t="n"/>
+      <c r="V25" s="19" t="n"/>
+      <c r="W25" s="19" t="n"/>
+      <c r="X25" s="19" t="n"/>
+      <c r="Y25" s="19" t="n"/>
+      <c r="Z25" s="19" t="n"/>
     </row>
     <row r="26">
       <c r="A26">
         <f>IF(Accounts!A26="","",Accounts!A26)</f>
         <v/>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="22">
         <f>IF(Accounts!B26="","",Accounts!B26)</f>
         <v/>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="18" t="n"/>
-      <c r="I26" s="18" t="n"/>
-      <c r="J26" s="18" t="n"/>
-      <c r="K26" s="18" t="n"/>
-      <c r="L26" s="18" t="n"/>
-      <c r="M26" s="18" t="n"/>
-      <c r="N26" s="18" t="n"/>
-      <c r="O26" s="18" t="n"/>
-      <c r="P26" s="18" t="n"/>
-      <c r="Q26" s="18" t="n"/>
-      <c r="R26" s="18" t="n"/>
-      <c r="S26" s="18" t="n"/>
-      <c r="T26" s="18" t="n"/>
-      <c r="U26" s="18" t="n"/>
-      <c r="V26" s="18" t="n"/>
-      <c r="W26" s="18" t="n"/>
-      <c r="X26" s="18" t="n"/>
-      <c r="Y26" s="18" t="n"/>
-      <c r="Z26" s="18" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19" t="n"/>
+      <c r="M26" s="19" t="n"/>
+      <c r="N26" s="19" t="n"/>
+      <c r="O26" s="19" t="n"/>
+      <c r="P26" s="19" t="n"/>
+      <c r="Q26" s="19" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
+      <c r="T26" s="19" t="n"/>
+      <c r="U26" s="19" t="n"/>
+      <c r="V26" s="19" t="n"/>
+      <c r="W26" s="19" t="n"/>
+      <c r="X26" s="19" t="n"/>
+      <c r="Y26" s="19" t="n"/>
+      <c r="Z26" s="19" t="n"/>
     </row>
     <row r="27">
       <c r="A27">
         <f>IF(Accounts!A27="","",Accounts!A27)</f>
         <v/>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="22">
         <f>IF(Accounts!B27="","",Accounts!B27)</f>
         <v/>
       </c>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="M27" s="18" t="n"/>
-      <c r="N27" s="18" t="n"/>
-      <c r="O27" s="18" t="n"/>
-      <c r="P27" s="18" t="n"/>
-      <c r="Q27" s="18" t="n"/>
-      <c r="R27" s="18" t="n"/>
-      <c r="S27" s="18" t="n"/>
-      <c r="T27" s="18" t="n"/>
-      <c r="U27" s="18" t="n"/>
-      <c r="V27" s="18" t="n"/>
-      <c r="W27" s="18" t="n"/>
-      <c r="X27" s="18" t="n"/>
-      <c r="Y27" s="18" t="n"/>
-      <c r="Z27" s="18" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="19" t="n"/>
+      <c r="I27" s="19" t="n"/>
+      <c r="J27" s="19" t="n"/>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="19" t="n"/>
+      <c r="O27" s="19" t="n"/>
+      <c r="P27" s="19" t="n"/>
+      <c r="Q27" s="19" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
+      <c r="T27" s="19" t="n"/>
+      <c r="U27" s="19" t="n"/>
+      <c r="V27" s="19" t="n"/>
+      <c r="W27" s="19" t="n"/>
+      <c r="X27" s="19" t="n"/>
+      <c r="Y27" s="19" t="n"/>
+      <c r="Z27" s="19" t="n"/>
     </row>
     <row r="28">
       <c r="A28">
         <f>IF(Accounts!A28="","",Accounts!A28)</f>
         <v/>
       </c>
-      <c r="B28" s="21">
+      <c r="B28" s="22">
         <f>IF(Accounts!B28="","",Accounts!B28)</f>
         <v/>
       </c>
-      <c r="C28" s="18" t="n"/>
-      <c r="D28" s="18" t="n"/>
-      <c r="E28" s="18" t="n"/>
-      <c r="F28" s="18" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="18" t="n"/>
-      <c r="I28" s="18" t="n"/>
-      <c r="J28" s="18" t="n"/>
-      <c r="K28" s="18" t="n"/>
-      <c r="L28" s="18" t="n"/>
-      <c r="M28" s="18" t="n"/>
-      <c r="N28" s="18" t="n"/>
-      <c r="O28" s="18" t="n"/>
-      <c r="P28" s="18" t="n"/>
-      <c r="Q28" s="18" t="n"/>
-      <c r="R28" s="18" t="n"/>
-      <c r="S28" s="18" t="n"/>
-      <c r="T28" s="18" t="n"/>
-      <c r="U28" s="18" t="n"/>
-      <c r="V28" s="18" t="n"/>
-      <c r="W28" s="18" t="n"/>
-      <c r="X28" s="18" t="n"/>
-      <c r="Y28" s="18" t="n"/>
-      <c r="Z28" s="18" t="n"/>
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19" t="n"/>
+      <c r="M28" s="19" t="n"/>
+      <c r="N28" s="19" t="n"/>
+      <c r="O28" s="19" t="n"/>
+      <c r="P28" s="19" t="n"/>
+      <c r="Q28" s="19" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
+      <c r="T28" s="19" t="n"/>
+      <c r="U28" s="19" t="n"/>
+      <c r="V28" s="19" t="n"/>
+      <c r="W28" s="19" t="n"/>
+      <c r="X28" s="19" t="n"/>
+      <c r="Y28" s="19" t="n"/>
+      <c r="Z28" s="19" t="n"/>
     </row>
     <row r="29">
       <c r="A29">
         <f>IF(Accounts!A29="","",Accounts!A29)</f>
         <v/>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="22">
         <f>IF(Accounts!B29="","",Accounts!B29)</f>
         <v/>
       </c>
-      <c r="C29" s="18" t="n"/>
-      <c r="D29" s="18" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="18" t="n"/>
-      <c r="I29" s="18" t="n"/>
-      <c r="J29" s="18" t="n"/>
-      <c r="K29" s="18" t="n"/>
-      <c r="L29" s="18" t="n"/>
-      <c r="M29" s="18" t="n"/>
-      <c r="N29" s="18" t="n"/>
-      <c r="O29" s="18" t="n"/>
-      <c r="P29" s="18" t="n"/>
-      <c r="Q29" s="18" t="n"/>
-      <c r="R29" s="18" t="n"/>
-      <c r="S29" s="18" t="n"/>
-      <c r="T29" s="18" t="n"/>
-      <c r="U29" s="18" t="n"/>
-      <c r="V29" s="18" t="n"/>
-      <c r="W29" s="18" t="n"/>
-      <c r="X29" s="18" t="n"/>
-      <c r="Y29" s="18" t="n"/>
-      <c r="Z29" s="18" t="n"/>
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="19" t="n"/>
+      <c r="I29" s="19" t="n"/>
+      <c r="J29" s="19" t="n"/>
+      <c r="K29" s="19" t="n"/>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="19" t="n"/>
+      <c r="O29" s="19" t="n"/>
+      <c r="P29" s="19" t="n"/>
+      <c r="Q29" s="19" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
+      <c r="T29" s="19" t="n"/>
+      <c r="U29" s="19" t="n"/>
+      <c r="V29" s="19" t="n"/>
+      <c r="W29" s="19" t="n"/>
+      <c r="X29" s="19" t="n"/>
+      <c r="Y29" s="19" t="n"/>
+      <c r="Z29" s="19" t="n"/>
     </row>
     <row r="30">
       <c r="A30">
         <f>IF(Accounts!A30="","",Accounts!A30)</f>
         <v/>
       </c>
-      <c r="B30" s="21">
+      <c r="B30" s="22">
         <f>IF(Accounts!B30="","",Accounts!B30)</f>
         <v/>
       </c>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="18" t="n"/>
-      <c r="K30" s="18" t="n"/>
-      <c r="L30" s="18" t="n"/>
-      <c r="M30" s="18" t="n"/>
-      <c r="N30" s="18" t="n"/>
-      <c r="O30" s="18" t="n"/>
-      <c r="P30" s="18" t="n"/>
-      <c r="Q30" s="18" t="n"/>
-      <c r="R30" s="18" t="n"/>
-      <c r="S30" s="18" t="n"/>
-      <c r="T30" s="18" t="n"/>
-      <c r="U30" s="18" t="n"/>
-      <c r="V30" s="18" t="n"/>
-      <c r="W30" s="18" t="n"/>
-      <c r="X30" s="18" t="n"/>
-      <c r="Y30" s="18" t="n"/>
-      <c r="Z30" s="18" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+      <c r="O30" s="19" t="n"/>
+      <c r="P30" s="19" t="n"/>
+      <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
+      <c r="T30" s="19" t="n"/>
+      <c r="U30" s="19" t="n"/>
+      <c r="V30" s="19" t="n"/>
+      <c r="W30" s="19" t="n"/>
+      <c r="X30" s="19" t="n"/>
+      <c r="Y30" s="19" t="n"/>
+      <c r="Z30" s="19" t="n"/>
     </row>
     <row r="31">
       <c r="A31">
         <f>IF(Accounts!A31="","",Accounts!A31)</f>
         <v/>
       </c>
-      <c r="B31" s="21">
+      <c r="B31" s="22">
         <f>IF(Accounts!B31="","",Accounts!B31)</f>
         <v/>
       </c>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="18" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="18" t="n"/>
-      <c r="L31" s="18" t="n"/>
-      <c r="M31" s="18" t="n"/>
-      <c r="N31" s="18" t="n"/>
-      <c r="O31" s="18" t="n"/>
-      <c r="P31" s="18" t="n"/>
-      <c r="Q31" s="18" t="n"/>
-      <c r="R31" s="18" t="n"/>
-      <c r="S31" s="18" t="n"/>
-      <c r="T31" s="18" t="n"/>
-      <c r="U31" s="18" t="n"/>
-      <c r="V31" s="18" t="n"/>
-      <c r="W31" s="18" t="n"/>
-      <c r="X31" s="18" t="n"/>
-      <c r="Y31" s="18" t="n"/>
-      <c r="Z31" s="18" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="19" t="n"/>
+      <c r="O31" s="19" t="n"/>
+      <c r="P31" s="19" t="n"/>
+      <c r="Q31" s="19" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
+      <c r="T31" s="19" t="n"/>
+      <c r="U31" s="19" t="n"/>
+      <c r="V31" s="19" t="n"/>
+      <c r="W31" s="19" t="n"/>
+      <c r="X31" s="19" t="n"/>
+      <c r="Y31" s="19" t="n"/>
+      <c r="Z31" s="19" t="n"/>
     </row>
     <row r="32">
       <c r="A32">
         <f>IF(Accounts!A32="","",Accounts!A32)</f>
         <v/>
       </c>
-      <c r="B32" s="21">
+      <c r="B32" s="22">
         <f>IF(Accounts!B32="","",Accounts!B32)</f>
         <v/>
       </c>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="18" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="18" t="n"/>
-      <c r="I32" s="18" t="n"/>
-      <c r="J32" s="18" t="n"/>
-      <c r="K32" s="18" t="n"/>
-      <c r="L32" s="18" t="n"/>
-      <c r="M32" s="18" t="n"/>
-      <c r="N32" s="18" t="n"/>
-      <c r="O32" s="18" t="n"/>
-      <c r="P32" s="18" t="n"/>
-      <c r="Q32" s="18" t="n"/>
-      <c r="R32" s="18" t="n"/>
-      <c r="S32" s="18" t="n"/>
-      <c r="T32" s="18" t="n"/>
-      <c r="U32" s="18" t="n"/>
-      <c r="V32" s="18" t="n"/>
-      <c r="W32" s="18" t="n"/>
-      <c r="X32" s="18" t="n"/>
-      <c r="Y32" s="18" t="n"/>
-      <c r="Z32" s="18" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="n"/>
+      <c r="H32" s="19" t="n"/>
+      <c r="I32" s="19" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19" t="n"/>
+      <c r="M32" s="19" t="n"/>
+      <c r="N32" s="19" t="n"/>
+      <c r="O32" s="19" t="n"/>
+      <c r="P32" s="19" t="n"/>
+      <c r="Q32" s="19" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
+      <c r="T32" s="19" t="n"/>
+      <c r="U32" s="19" t="n"/>
+      <c r="V32" s="19" t="n"/>
+      <c r="W32" s="19" t="n"/>
+      <c r="X32" s="19" t="n"/>
+      <c r="Y32" s="19" t="n"/>
+      <c r="Z32" s="19" t="n"/>
     </row>
     <row r="33">
       <c r="A33">
         <f>IF(Accounts!A33="","",Accounts!A33)</f>
         <v/>
       </c>
-      <c r="B33" s="21">
+      <c r="B33" s="22">
         <f>IF(Accounts!B33="","",Accounts!B33)</f>
         <v/>
       </c>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="18" t="n"/>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
-      <c r="G33" s="18" t="n"/>
-      <c r="H33" s="18" t="n"/>
-      <c r="I33" s="18" t="n"/>
-      <c r="J33" s="18" t="n"/>
-      <c r="K33" s="18" t="n"/>
-      <c r="L33" s="18" t="n"/>
-      <c r="M33" s="18" t="n"/>
-      <c r="N33" s="18" t="n"/>
-      <c r="O33" s="18" t="n"/>
-      <c r="P33" s="18" t="n"/>
-      <c r="Q33" s="18" t="n"/>
-      <c r="R33" s="18" t="n"/>
-      <c r="S33" s="18" t="n"/>
-      <c r="T33" s="18" t="n"/>
-      <c r="U33" s="18" t="n"/>
-      <c r="V33" s="18" t="n"/>
-      <c r="W33" s="18" t="n"/>
-      <c r="X33" s="18" t="n"/>
-      <c r="Y33" s="18" t="n"/>
-      <c r="Z33" s="18" t="n"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="19" t="n"/>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n"/>
+      <c r="N33" s="19" t="n"/>
+      <c r="O33" s="19" t="n"/>
+      <c r="P33" s="19" t="n"/>
+      <c r="Q33" s="19" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
+      <c r="T33" s="19" t="n"/>
+      <c r="U33" s="19" t="n"/>
+      <c r="V33" s="19" t="n"/>
+      <c r="W33" s="19" t="n"/>
+      <c r="X33" s="19" t="n"/>
+      <c r="Y33" s="19" t="n"/>
+      <c r="Z33" s="19" t="n"/>
     </row>
     <row r="34">
       <c r="A34">
         <f>IF(Accounts!A34="","",Accounts!A34)</f>
         <v/>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="22">
         <f>IF(Accounts!B34="","",Accounts!B34)</f>
         <v/>
       </c>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="18" t="n"/>
-      <c r="E34" s="18" t="n"/>
-      <c r="F34" s="18" t="n"/>
-      <c r="G34" s="18" t="n"/>
-      <c r="H34" s="18" t="n"/>
-      <c r="I34" s="18" t="n"/>
-      <c r="J34" s="18" t="n"/>
-      <c r="K34" s="18" t="n"/>
-      <c r="L34" s="18" t="n"/>
-      <c r="M34" s="18" t="n"/>
-      <c r="N34" s="18" t="n"/>
-      <c r="O34" s="18" t="n"/>
-      <c r="P34" s="18" t="n"/>
-      <c r="Q34" s="18" t="n"/>
-      <c r="R34" s="18" t="n"/>
-      <c r="S34" s="18" t="n"/>
-      <c r="T34" s="18" t="n"/>
-      <c r="U34" s="18" t="n"/>
-      <c r="V34" s="18" t="n"/>
-      <c r="W34" s="18" t="n"/>
-      <c r="X34" s="18" t="n"/>
-      <c r="Y34" s="18" t="n"/>
-      <c r="Z34" s="18" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="n"/>
+      <c r="H34" s="19" t="n"/>
+      <c r="I34" s="19" t="n"/>
+      <c r="J34" s="19" t="n"/>
+      <c r="K34" s="19" t="n"/>
+      <c r="L34" s="19" t="n"/>
+      <c r="M34" s="19" t="n"/>
+      <c r="N34" s="19" t="n"/>
+      <c r="O34" s="19" t="n"/>
+      <c r="P34" s="19" t="n"/>
+      <c r="Q34" s="19" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
+      <c r="T34" s="19" t="n"/>
+      <c r="U34" s="19" t="n"/>
+      <c r="V34" s="19" t="n"/>
+      <c r="W34" s="19" t="n"/>
+      <c r="X34" s="19" t="n"/>
+      <c r="Y34" s="19" t="n"/>
+      <c r="Z34" s="19" t="n"/>
     </row>
     <row r="35">
       <c r="A35">
         <f>IF(Accounts!A35="","",Accounts!A35)</f>
         <v/>
       </c>
-      <c r="B35" s="21">
+      <c r="B35" s="22">
         <f>IF(Accounts!B35="","",Accounts!B35)</f>
         <v/>
       </c>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="18" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18" t="n"/>
-      <c r="G35" s="18" t="n"/>
-      <c r="H35" s="18" t="n"/>
-      <c r="I35" s="18" t="n"/>
-      <c r="J35" s="18" t="n"/>
-      <c r="K35" s="18" t="n"/>
-      <c r="L35" s="18" t="n"/>
-      <c r="M35" s="18" t="n"/>
-      <c r="N35" s="18" t="n"/>
-      <c r="O35" s="18" t="n"/>
-      <c r="P35" s="18" t="n"/>
-      <c r="Q35" s="18" t="n"/>
-      <c r="R35" s="18" t="n"/>
-      <c r="S35" s="18" t="n"/>
-      <c r="T35" s="18" t="n"/>
-      <c r="U35" s="18" t="n"/>
-      <c r="V35" s="18" t="n"/>
-      <c r="W35" s="18" t="n"/>
-      <c r="X35" s="18" t="n"/>
-      <c r="Y35" s="18" t="n"/>
-      <c r="Z35" s="18" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="19" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="19" t="n"/>
+      <c r="O35" s="19" t="n"/>
+      <c r="P35" s="19" t="n"/>
+      <c r="Q35" s="19" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
+      <c r="T35" s="19" t="n"/>
+      <c r="U35" s="19" t="n"/>
+      <c r="V35" s="19" t="n"/>
+      <c r="W35" s="19" t="n"/>
+      <c r="X35" s="19" t="n"/>
+      <c r="Y35" s="19" t="n"/>
+      <c r="Z35" s="19" t="n"/>
     </row>
     <row r="36">
       <c r="A36">
         <f>IF(Accounts!A36="","",Accounts!A36)</f>
         <v/>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="22">
         <f>IF(Accounts!B36="","",Accounts!B36)</f>
         <v/>
       </c>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
-      <c r="I36" s="18" t="n"/>
-      <c r="J36" s="18" t="n"/>
-      <c r="K36" s="18" t="n"/>
-      <c r="L36" s="18" t="n"/>
-      <c r="M36" s="18" t="n"/>
-      <c r="N36" s="18" t="n"/>
-      <c r="O36" s="18" t="n"/>
-      <c r="P36" s="18" t="n"/>
-      <c r="Q36" s="18" t="n"/>
-      <c r="R36" s="18" t="n"/>
-      <c r="S36" s="18" t="n"/>
-      <c r="T36" s="18" t="n"/>
-      <c r="U36" s="18" t="n"/>
-      <c r="V36" s="18" t="n"/>
-      <c r="W36" s="18" t="n"/>
-      <c r="X36" s="18" t="n"/>
-      <c r="Y36" s="18" t="n"/>
-      <c r="Z36" s="18" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="n"/>
+      <c r="M36" s="19" t="n"/>
+      <c r="N36" s="19" t="n"/>
+      <c r="O36" s="19" t="n"/>
+      <c r="P36" s="19" t="n"/>
+      <c r="Q36" s="19" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
+      <c r="T36" s="19" t="n"/>
+      <c r="U36" s="19" t="n"/>
+      <c r="V36" s="19" t="n"/>
+      <c r="W36" s="19" t="n"/>
+      <c r="X36" s="19" t="n"/>
+      <c r="Y36" s="19" t="n"/>
+      <c r="Z36" s="19" t="n"/>
     </row>
     <row r="37">
       <c r="A37">
         <f>IF(Accounts!A37="","",Accounts!A37)</f>
         <v/>
       </c>
-      <c r="B37" s="21">
+      <c r="B37" s="22">
         <f>IF(Accounts!B37="","",Accounts!B37)</f>
         <v/>
       </c>
-      <c r="C37" s="18" t="n"/>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="18" t="n"/>
-      <c r="H37" s="18" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="18" t="n"/>
-      <c r="L37" s="18" t="n"/>
-      <c r="M37" s="18" t="n"/>
-      <c r="N37" s="18" t="n"/>
-      <c r="O37" s="18" t="n"/>
-      <c r="P37" s="18" t="n"/>
-      <c r="Q37" s="18" t="n"/>
-      <c r="R37" s="18" t="n"/>
-      <c r="S37" s="18" t="n"/>
-      <c r="T37" s="18" t="n"/>
-      <c r="U37" s="18" t="n"/>
-      <c r="V37" s="18" t="n"/>
-      <c r="W37" s="18" t="n"/>
-      <c r="X37" s="18" t="n"/>
-      <c r="Y37" s="18" t="n"/>
-      <c r="Z37" s="18" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
+      <c r="I37" s="19" t="n"/>
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="19" t="n"/>
+      <c r="N37" s="19" t="n"/>
+      <c r="O37" s="19" t="n"/>
+      <c r="P37" s="19" t="n"/>
+      <c r="Q37" s="19" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
+      <c r="T37" s="19" t="n"/>
+      <c r="U37" s="19" t="n"/>
+      <c r="V37" s="19" t="n"/>
+      <c r="W37" s="19" t="n"/>
+      <c r="X37" s="19" t="n"/>
+      <c r="Y37" s="19" t="n"/>
+      <c r="Z37" s="19" t="n"/>
     </row>
     <row r="38">
       <c r="A38">
         <f>IF(Accounts!A38="","",Accounts!A38)</f>
         <v/>
       </c>
-      <c r="B38" s="21">
+      <c r="B38" s="22">
         <f>IF(Accounts!B38="","",Accounts!B38)</f>
         <v/>
       </c>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18" t="n"/>
-      <c r="G38" s="18" t="n"/>
-      <c r="H38" s="18" t="n"/>
-      <c r="I38" s="18" t="n"/>
-      <c r="J38" s="18" t="n"/>
-      <c r="K38" s="18" t="n"/>
-      <c r="L38" s="18" t="n"/>
-      <c r="M38" s="18" t="n"/>
-      <c r="N38" s="18" t="n"/>
-      <c r="O38" s="18" t="n"/>
-      <c r="P38" s="18" t="n"/>
-      <c r="Q38" s="18" t="n"/>
-      <c r="R38" s="18" t="n"/>
-      <c r="S38" s="18" t="n"/>
-      <c r="T38" s="18" t="n"/>
-      <c r="U38" s="18" t="n"/>
-      <c r="V38" s="18" t="n"/>
-      <c r="W38" s="18" t="n"/>
-      <c r="X38" s="18" t="n"/>
-      <c r="Y38" s="18" t="n"/>
-      <c r="Z38" s="18" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="19" t="n"/>
+      <c r="H38" s="19" t="n"/>
+      <c r="I38" s="19" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="19" t="n"/>
+      <c r="M38" s="19" t="n"/>
+      <c r="N38" s="19" t="n"/>
+      <c r="O38" s="19" t="n"/>
+      <c r="P38" s="19" t="n"/>
+      <c r="Q38" s="19" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
+      <c r="T38" s="19" t="n"/>
+      <c r="U38" s="19" t="n"/>
+      <c r="V38" s="19" t="n"/>
+      <c r="W38" s="19" t="n"/>
+      <c r="X38" s="19" t="n"/>
+      <c r="Y38" s="19" t="n"/>
+      <c r="Z38" s="19" t="n"/>
     </row>
     <row r="39">
       <c r="A39">
         <f>IF(Accounts!A39="","",Accounts!A39)</f>
         <v/>
       </c>
-      <c r="B39" s="21">
+      <c r="B39" s="22">
         <f>IF(Accounts!B39="","",Accounts!B39)</f>
         <v/>
       </c>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="18" t="n"/>
-      <c r="F39" s="18" t="n"/>
-      <c r="G39" s="18" t="n"/>
-      <c r="H39" s="18" t="n"/>
-      <c r="I39" s="18" t="n"/>
-      <c r="J39" s="18" t="n"/>
-      <c r="K39" s="18" t="n"/>
-      <c r="L39" s="18" t="n"/>
-      <c r="M39" s="18" t="n"/>
-      <c r="N39" s="18" t="n"/>
-      <c r="O39" s="18" t="n"/>
-      <c r="P39" s="18" t="n"/>
-      <c r="Q39" s="18" t="n"/>
-      <c r="R39" s="18" t="n"/>
-      <c r="S39" s="18" t="n"/>
-      <c r="T39" s="18" t="n"/>
-      <c r="U39" s="18" t="n"/>
-      <c r="V39" s="18" t="n"/>
-      <c r="W39" s="18" t="n"/>
-      <c r="X39" s="18" t="n"/>
-      <c r="Y39" s="18" t="n"/>
-      <c r="Z39" s="18" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+      <c r="O39" s="19" t="n"/>
+      <c r="P39" s="19" t="n"/>
+      <c r="Q39" s="19" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
+      <c r="T39" s="19" t="n"/>
+      <c r="U39" s="19" t="n"/>
+      <c r="V39" s="19" t="n"/>
+      <c r="W39" s="19" t="n"/>
+      <c r="X39" s="19" t="n"/>
+      <c r="Y39" s="19" t="n"/>
+      <c r="Z39" s="19" t="n"/>
     </row>
     <row r="40">
       <c r="A40">
         <f>IF(Accounts!A40="","",Accounts!A40)</f>
         <v/>
       </c>
-      <c r="B40" s="21">
+      <c r="B40" s="22">
         <f>IF(Accounts!B40="","",Accounts!B40)</f>
         <v/>
       </c>
-      <c r="C40" s="18" t="n"/>
-      <c r="D40" s="18" t="n"/>
-      <c r="E40" s="18" t="n"/>
-      <c r="F40" s="18" t="n"/>
-      <c r="G40" s="18" t="n"/>
-      <c r="H40" s="18" t="n"/>
-      <c r="I40" s="18" t="n"/>
-      <c r="J40" s="18" t="n"/>
-      <c r="K40" s="18" t="n"/>
-      <c r="L40" s="18" t="n"/>
-      <c r="M40" s="18" t="n"/>
-      <c r="N40" s="18" t="n"/>
-      <c r="O40" s="18" t="n"/>
-      <c r="P40" s="18" t="n"/>
-      <c r="Q40" s="18" t="n"/>
-      <c r="R40" s="18" t="n"/>
-      <c r="S40" s="18" t="n"/>
-      <c r="T40" s="18" t="n"/>
-      <c r="U40" s="18" t="n"/>
-      <c r="V40" s="18" t="n"/>
-      <c r="W40" s="18" t="n"/>
-      <c r="X40" s="18" t="n"/>
-      <c r="Y40" s="18" t="n"/>
-      <c r="Z40" s="18" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="19" t="n"/>
+      <c r="I40" s="19" t="n"/>
+      <c r="J40" s="19" t="n"/>
+      <c r="K40" s="19" t="n"/>
+      <c r="L40" s="19" t="n"/>
+      <c r="M40" s="19" t="n"/>
+      <c r="N40" s="19" t="n"/>
+      <c r="O40" s="19" t="n"/>
+      <c r="P40" s="19" t="n"/>
+      <c r="Q40" s="19" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
+      <c r="T40" s="19" t="n"/>
+      <c r="U40" s="19" t="n"/>
+      <c r="V40" s="19" t="n"/>
+      <c r="W40" s="19" t="n"/>
+      <c r="X40" s="19" t="n"/>
+      <c r="Y40" s="19" t="n"/>
+      <c r="Z40" s="19" t="n"/>
     </row>
     <row r="41">
       <c r="A41">
         <f>IF(Accounts!A41="","",Accounts!A41)</f>
         <v/>
       </c>
-      <c r="B41" s="21">
+      <c r="B41" s="22">
         <f>IF(Accounts!B41="","",Accounts!B41)</f>
         <v/>
       </c>
-      <c r="C41" s="18" t="n"/>
-      <c r="D41" s="18" t="n"/>
-      <c r="E41" s="18" t="n"/>
-      <c r="F41" s="18" t="n"/>
-      <c r="G41" s="18" t="n"/>
-      <c r="H41" s="18" t="n"/>
-      <c r="I41" s="18" t="n"/>
-      <c r="J41" s="18" t="n"/>
-      <c r="K41" s="18" t="n"/>
-      <c r="L41" s="18" t="n"/>
-      <c r="M41" s="18" t="n"/>
-      <c r="N41" s="18" t="n"/>
-      <c r="O41" s="18" t="n"/>
-      <c r="P41" s="18" t="n"/>
-      <c r="Q41" s="18" t="n"/>
-      <c r="R41" s="18" t="n"/>
-      <c r="S41" s="18" t="n"/>
-      <c r="T41" s="18" t="n"/>
-      <c r="U41" s="18" t="n"/>
-      <c r="V41" s="18" t="n"/>
-      <c r="W41" s="18" t="n"/>
-      <c r="X41" s="18" t="n"/>
-      <c r="Y41" s="18" t="n"/>
-      <c r="Z41" s="18" t="n"/>
+      <c r="C41" s="19" t="n"/>
+      <c r="D41" s="19" t="n"/>
+      <c r="E41" s="19" t="n"/>
+      <c r="F41" s="19" t="n"/>
+      <c r="G41" s="19" t="n"/>
+      <c r="H41" s="19" t="n"/>
+      <c r="I41" s="19" t="n"/>
+      <c r="J41" s="19" t="n"/>
+      <c r="K41" s="19" t="n"/>
+      <c r="L41" s="19" t="n"/>
+      <c r="M41" s="19" t="n"/>
+      <c r="N41" s="19" t="n"/>
+      <c r="O41" s="19" t="n"/>
+      <c r="P41" s="19" t="n"/>
+      <c r="Q41" s="19" t="n"/>
+      <c r="R41" s="19" t="n"/>
+      <c r="S41" s="19" t="n"/>
+      <c r="T41" s="19" t="n"/>
+      <c r="U41" s="19" t="n"/>
+      <c r="V41" s="19" t="n"/>
+      <c r="W41" s="19" t="n"/>
+      <c r="X41" s="19" t="n"/>
+      <c r="Y41" s="19" t="n"/>
+      <c r="Z41" s="19" t="n"/>
     </row>
     <row r="42">
       <c r="A42">
         <f>IF(Accounts!A42="","",Accounts!A42)</f>
         <v/>
       </c>
-      <c r="B42" s="21">
+      <c r="B42" s="22">
         <f>IF(Accounts!B42="","",Accounts!B42)</f>
         <v/>
       </c>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="18" t="n"/>
-      <c r="F42" s="18" t="n"/>
-      <c r="G42" s="18" t="n"/>
-      <c r="H42" s="18" t="n"/>
-      <c r="I42" s="18" t="n"/>
-      <c r="J42" s="18" t="n"/>
-      <c r="K42" s="18" t="n"/>
-      <c r="L42" s="18" t="n"/>
-      <c r="M42" s="18" t="n"/>
-      <c r="N42" s="18" t="n"/>
-      <c r="O42" s="18" t="n"/>
-      <c r="P42" s="18" t="n"/>
-      <c r="Q42" s="18" t="n"/>
-      <c r="R42" s="18" t="n"/>
-      <c r="S42" s="18" t="n"/>
-      <c r="T42" s="18" t="n"/>
-      <c r="U42" s="18" t="n"/>
-      <c r="V42" s="18" t="n"/>
-      <c r="W42" s="18" t="n"/>
-      <c r="X42" s="18" t="n"/>
-      <c r="Y42" s="18" t="n"/>
-      <c r="Z42" s="18" t="n"/>
+      <c r="C42" s="19" t="n"/>
+      <c r="D42" s="19" t="n"/>
+      <c r="E42" s="19" t="n"/>
+      <c r="F42" s="19" t="n"/>
+      <c r="G42" s="19" t="n"/>
+      <c r="H42" s="19" t="n"/>
+      <c r="I42" s="19" t="n"/>
+      <c r="J42" s="19" t="n"/>
+      <c r="K42" s="19" t="n"/>
+      <c r="L42" s="19" t="n"/>
+      <c r="M42" s="19" t="n"/>
+      <c r="N42" s="19" t="n"/>
+      <c r="O42" s="19" t="n"/>
+      <c r="P42" s="19" t="n"/>
+      <c r="Q42" s="19" t="n"/>
+      <c r="R42" s="19" t="n"/>
+      <c r="S42" s="19" t="n"/>
+      <c r="T42" s="19" t="n"/>
+      <c r="U42" s="19" t="n"/>
+      <c r="V42" s="19" t="n"/>
+      <c r="W42" s="19" t="n"/>
+      <c r="X42" s="19" t="n"/>
+      <c r="Y42" s="19" t="n"/>
+      <c r="Z42" s="19" t="n"/>
     </row>
     <row r="43">
       <c r="A43">
         <f>IF(Accounts!A43="","",Accounts!A43)</f>
         <v/>
       </c>
-      <c r="B43" s="21">
+      <c r="B43" s="22">
         <f>IF(Accounts!B43="","",Accounts!B43)</f>
         <v/>
       </c>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="18" t="n"/>
-      <c r="G43" s="18" t="n"/>
-      <c r="H43" s="18" t="n"/>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18" t="n"/>
-      <c r="K43" s="18" t="n"/>
-      <c r="L43" s="18" t="n"/>
-      <c r="M43" s="18" t="n"/>
-      <c r="N43" s="18" t="n"/>
-      <c r="O43" s="18" t="n"/>
-      <c r="P43" s="18" t="n"/>
-      <c r="Q43" s="18" t="n"/>
-      <c r="R43" s="18" t="n"/>
-      <c r="S43" s="18" t="n"/>
-      <c r="T43" s="18" t="n"/>
-      <c r="U43" s="18" t="n"/>
-      <c r="V43" s="18" t="n"/>
-      <c r="W43" s="18" t="n"/>
-      <c r="X43" s="18" t="n"/>
-      <c r="Y43" s="18" t="n"/>
-      <c r="Z43" s="18" t="n"/>
+      <c r="C43" s="19" t="n"/>
+      <c r="D43" s="19" t="n"/>
+      <c r="E43" s="19" t="n"/>
+      <c r="F43" s="19" t="n"/>
+      <c r="G43" s="19" t="n"/>
+      <c r="H43" s="19" t="n"/>
+      <c r="I43" s="19" t="n"/>
+      <c r="J43" s="19" t="n"/>
+      <c r="K43" s="19" t="n"/>
+      <c r="L43" s="19" t="n"/>
+      <c r="M43" s="19" t="n"/>
+      <c r="N43" s="19" t="n"/>
+      <c r="O43" s="19" t="n"/>
+      <c r="P43" s="19" t="n"/>
+      <c r="Q43" s="19" t="n"/>
+      <c r="R43" s="19" t="n"/>
+      <c r="S43" s="19" t="n"/>
+      <c r="T43" s="19" t="n"/>
+      <c r="U43" s="19" t="n"/>
+      <c r="V43" s="19" t="n"/>
+      <c r="W43" s="19" t="n"/>
+      <c r="X43" s="19" t="n"/>
+      <c r="Y43" s="19" t="n"/>
+      <c r="Z43" s="19" t="n"/>
     </row>
     <row r="44">
       <c r="A44">
         <f>IF(Accounts!A44="","",Accounts!A44)</f>
         <v/>
       </c>
-      <c r="B44" s="21">
+      <c r="B44" s="22">
         <f>IF(Accounts!B44="","",Accounts!B44)</f>
         <v/>
       </c>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="18" t="n"/>
-      <c r="G44" s="18" t="n"/>
-      <c r="H44" s="18" t="n"/>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18" t="n"/>
-      <c r="K44" s="18" t="n"/>
-      <c r="L44" s="18" t="n"/>
-      <c r="M44" s="18" t="n"/>
-      <c r="N44" s="18" t="n"/>
-      <c r="O44" s="18" t="n"/>
-      <c r="P44" s="18" t="n"/>
-      <c r="Q44" s="18" t="n"/>
-      <c r="R44" s="18" t="n"/>
-      <c r="S44" s="18" t="n"/>
-      <c r="T44" s="18" t="n"/>
-      <c r="U44" s="18" t="n"/>
-      <c r="V44" s="18" t="n"/>
-      <c r="W44" s="18" t="n"/>
-      <c r="X44" s="18" t="n"/>
-      <c r="Y44" s="18" t="n"/>
-      <c r="Z44" s="18" t="n"/>
+      <c r="C44" s="19" t="n"/>
+      <c r="D44" s="19" t="n"/>
+      <c r="E44" s="19" t="n"/>
+      <c r="F44" s="19" t="n"/>
+      <c r="G44" s="19" t="n"/>
+      <c r="H44" s="19" t="n"/>
+      <c r="I44" s="19" t="n"/>
+      <c r="J44" s="19" t="n"/>
+      <c r="K44" s="19" t="n"/>
+      <c r="L44" s="19" t="n"/>
+      <c r="M44" s="19" t="n"/>
+      <c r="N44" s="19" t="n"/>
+      <c r="O44" s="19" t="n"/>
+      <c r="P44" s="19" t="n"/>
+      <c r="Q44" s="19" t="n"/>
+      <c r="R44" s="19" t="n"/>
+      <c r="S44" s="19" t="n"/>
+      <c r="T44" s="19" t="n"/>
+      <c r="U44" s="19" t="n"/>
+      <c r="V44" s="19" t="n"/>
+      <c r="W44" s="19" t="n"/>
+      <c r="X44" s="19" t="n"/>
+      <c r="Y44" s="19" t="n"/>
+      <c r="Z44" s="19" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -3956,99 +3962,99 @@
         </is>
       </c>
       <c r="C50" s="14">
-        <f>IF(C$53=1,SUMIFS(C$5:C$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(C$53=1,SUMIFS(C$5:C$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="D50" s="14">
-        <f>IF(D$53=1,SUMIFS(D$5:D$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(D$53=1,SUMIFS(D$5:D$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="E50" s="14">
-        <f>IF(E$53=1,SUMIFS(E$5:E$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(E$53=1,SUMIFS(E$5:E$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="F50" s="14">
-        <f>IF(F$53=1,SUMIFS(F$5:F$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(F$53=1,SUMIFS(F$5:F$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="G50" s="14">
-        <f>IF(G$53=1,SUMIFS(G$5:G$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(G$53=1,SUMIFS(G$5:G$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="H50" s="14">
-        <f>IF(H$53=1,SUMIFS(H$5:H$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(H$53=1,SUMIFS(H$5:H$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="I50" s="14">
-        <f>IF(I$53=1,SUMIFS(I$5:I$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(I$53=1,SUMIFS(I$5:I$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="J50" s="14">
-        <f>IF(J$53=1,SUMIFS(J$5:J$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(J$53=1,SUMIFS(J$5:J$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="K50" s="14">
-        <f>IF(K$53=1,SUMIFS(K$5:K$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(K$53=1,SUMIFS(K$5:K$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="L50" s="14">
-        <f>IF(L$53=1,SUMIFS(L$5:L$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(L$53=1,SUMIFS(L$5:L$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="M50" s="14">
-        <f>IF(M$53=1,SUMIFS(M$5:M$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(M$53=1,SUMIFS(M$5:M$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="N50" s="14">
-        <f>IF(N$53=1,SUMIFS(N$5:N$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(N$53=1,SUMIFS(N$5:N$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="O50" s="14">
-        <f>IF(O$53=1,SUMIFS(O$5:O$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(O$53=1,SUMIFS(O$5:O$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="P50" s="14">
-        <f>IF(P$53=1,SUMIFS(P$5:P$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(P$53=1,SUMIFS(P$5:P$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Q50" s="14">
-        <f>IF(Q$53=1,SUMIFS(Q$5:Q$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(Q$53=1,SUMIFS(Q$5:Q$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="R50" s="14">
-        <f>IF(R$53=1,SUMIFS(R$5:R$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(R$53=1,SUMIFS(R$5:R$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="S50" s="14">
-        <f>IF(S$53=1,SUMIFS(S$5:S$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(S$53=1,SUMIFS(S$5:S$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="T50" s="14">
-        <f>IF(T$53=1,SUMIFS(T$5:T$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(T$53=1,SUMIFS(T$5:T$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="U50" s="14">
-        <f>IF(U$53=1,SUMIFS(U$5:U$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(U$53=1,SUMIFS(U$5:U$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="V50" s="14">
-        <f>IF(V$53=1,SUMIFS(V$5:V$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(V$53=1,SUMIFS(V$5:V$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="W50" s="14">
-        <f>IF(W$53=1,SUMIFS(W$5:W$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(W$53=1,SUMIFS(W$5:W$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="X50" s="14">
-        <f>IF(X$53=1,SUMIFS(X$5:X$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(X$53=1,SUMIFS(X$5:X$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Y50" s="14">
-        <f>IF(Y$53=1,SUMIFS(Y$5:Y$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(Y$53=1,SUMIFS(Y$5:Y$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Z50" s="14">
-        <f>IF(Z$53=1,SUMIFS(Z$5:Z$44,Accounts!$D$5:$D$44,"Yes"),"")</f>
+        <f>IF(Z$53=1,SUMIFS(Z$5:Z$44,Accounts!$C$5:$C$44,"Asset",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
     </row>
@@ -4059,99 +4065,99 @@
         </is>
       </c>
       <c r="C51" s="12">
-        <f>IF(C$53=1,C50-C48,"")</f>
+        <f>IF(C$53=1,C50-SUMIFS(C$5:C$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>IF(D$53=1,D50-D48,"")</f>
+        <f>IF(D$53=1,D50-SUMIFS(D$5:D$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>IF(E$53=1,E50-E48,"")</f>
+        <f>IF(E$53=1,E50-SUMIFS(E$5:E$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>IF(F$53=1,F50-F48,"")</f>
+        <f>IF(F$53=1,F50-SUMIFS(F$5:F$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="G51" s="12">
-        <f>IF(G$53=1,G50-G48,"")</f>
+        <f>IF(G$53=1,G50-SUMIFS(G$5:G$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="H51" s="12">
-        <f>IF(H$53=1,H50-H48,"")</f>
+        <f>IF(H$53=1,H50-SUMIFS(H$5:H$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="I51" s="12">
-        <f>IF(I$53=1,I50-I48,"")</f>
+        <f>IF(I$53=1,I50-SUMIFS(I$5:I$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="J51" s="12">
-        <f>IF(J$53=1,J50-J48,"")</f>
+        <f>IF(J$53=1,J50-SUMIFS(J$5:J$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="K51" s="12">
-        <f>IF(K$53=1,K50-K48,"")</f>
+        <f>IF(K$53=1,K50-SUMIFS(K$5:K$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="L51" s="12">
-        <f>IF(L$53=1,L50-L48,"")</f>
+        <f>IF(L$53=1,L50-SUMIFS(L$5:L$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="M51" s="12">
-        <f>IF(M$53=1,M50-M48,"")</f>
+        <f>IF(M$53=1,M50-SUMIFS(M$5:M$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="N51" s="12">
-        <f>IF(N$53=1,N50-N48,"")</f>
+        <f>IF(N$53=1,N50-SUMIFS(N$5:N$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="O51" s="12">
-        <f>IF(O$53=1,O50-O48,"")</f>
+        <f>IF(O$53=1,O50-SUMIFS(O$5:O$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="P51" s="12">
-        <f>IF(P$53=1,P50-P48,"")</f>
+        <f>IF(P$53=1,P50-SUMIFS(P$5:P$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Q51" s="12">
-        <f>IF(Q$53=1,Q50-Q48,"")</f>
+        <f>IF(Q$53=1,Q50-SUMIFS(Q$5:Q$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="R51" s="12">
-        <f>IF(R$53=1,R50-R48,"")</f>
+        <f>IF(R$53=1,R50-SUMIFS(R$5:R$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="S51" s="12">
-        <f>IF(S$53=1,S50-S48,"")</f>
+        <f>IF(S$53=1,S50-SUMIFS(S$5:S$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="T51" s="12">
-        <f>IF(T$53=1,T50-T48,"")</f>
+        <f>IF(T$53=1,T50-SUMIFS(T$5:T$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="U51" s="12">
-        <f>IF(U$53=1,U50-U48,"")</f>
+        <f>IF(U$53=1,U50-SUMIFS(U$5:U$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="V51" s="12">
-        <f>IF(V$53=1,V50-V48,"")</f>
+        <f>IF(V$53=1,V50-SUMIFS(V$5:V$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="W51" s="12">
-        <f>IF(W$53=1,W50-W48,"")</f>
+        <f>IF(W$53=1,W50-SUMIFS(W$5:W$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="X51" s="12">
-        <f>IF(X$53=1,X50-X48,"")</f>
+        <f>IF(X$53=1,X50-SUMIFS(X$5:X$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Y51" s="12">
-        <f>IF(Y$53=1,Y50-Y48,"")</f>
+        <f>IF(Y$53=1,Y50-SUMIFS(Y$5:Y$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
       <c r="Z51" s="12">
-        <f>IF(Z$53=1,Z50-Z48,"")</f>
+        <f>IF(Z$53=1,Z50-SUMIFS(Z$5:Z$44,Accounts!$C$5:$C$44,"Debt",Accounts!$D$5:$D$44,"Yes"),"")</f>
         <v/>
       </c>
     </row>
@@ -4269,99 +4275,99 @@
           <t>(1 = yes; used by Dashboard)</t>
         </is>
       </c>
-      <c r="C53" s="24">
+      <c r="C53" s="25">
         <f>IF(COUNT(C$5:C$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="D53" s="24">
+      <c r="D53" s="25">
         <f>IF(COUNT(D$5:D$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="E53" s="24">
+      <c r="E53" s="25">
         <f>IF(COUNT(E$5:E$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="F53" s="24">
+      <c r="F53" s="25">
         <f>IF(COUNT(F$5:F$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="G53" s="24">
+      <c r="G53" s="25">
         <f>IF(COUNT(G$5:G$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="H53" s="24">
+      <c r="H53" s="25">
         <f>IF(COUNT(H$5:H$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="I53" s="24">
+      <c r="I53" s="25">
         <f>IF(COUNT(I$5:I$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="J53" s="24">
+      <c r="J53" s="25">
         <f>IF(COUNT(J$5:J$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="K53" s="24">
+      <c r="K53" s="25">
         <f>IF(COUNT(K$5:K$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="L53" s="24">
+      <c r="L53" s="25">
         <f>IF(COUNT(L$5:L$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="M53" s="24">
+      <c r="M53" s="25">
         <f>IF(COUNT(M$5:M$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="N53" s="24">
+      <c r="N53" s="25">
         <f>IF(COUNT(N$5:N$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="O53" s="24">
+      <c r="O53" s="25">
         <f>IF(COUNT(O$5:O$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="P53" s="24">
+      <c r="P53" s="25">
         <f>IF(COUNT(P$5:P$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="Q53" s="24">
+      <c r="Q53" s="25">
         <f>IF(COUNT(Q$5:Q$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="R53" s="24">
+      <c r="R53" s="25">
         <f>IF(COUNT(R$5:R$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="S53" s="24">
+      <c r="S53" s="25">
         <f>IF(COUNT(S$5:S$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="T53" s="24">
+      <c r="T53" s="25">
         <f>IF(COUNT(T$5:T$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="U53" s="24">
+      <c r="U53" s="25">
         <f>IF(COUNT(U$5:U$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="V53" s="24">
+      <c r="V53" s="25">
         <f>IF(COUNT(V$5:V$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="W53" s="24">
+      <c r="W53" s="25">
         <f>IF(COUNT(W$5:W$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="X53" s="24">
+      <c r="X53" s="25">
         <f>IF(COUNT(X$5:X$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="Y53" s="24">
+      <c r="Y53" s="25">
         <f>IF(COUNT(Y$5:Y$44)&gt;0,1,"")</f>
         <v/>
       </c>
-      <c r="Z53" s="24">
+      <c r="Z53" s="25">
         <f>IF(COUNT(Z$5:Z$44)&gt;0,1,"")</f>
         <v/>
       </c>
@@ -4560,7 +4566,11 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n"/>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -4586,7 +4596,11 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n"/>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -4599,7 +4613,11 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="C16" s="15" t="n"/>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>